<commit_message>
Updated Work Log as part of Progress Report 2 submission
</commit_message>
<xml_diff>
--- a/DocumentsAndReports/worklog/WorkLog_DesmondChua_W26_4495_S2.xlsx
+++ b/DocumentsAndReports/worklog/WorkLog_DesmondChua_W26_4495_S2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d4f25ae689476683/Desmond_New/Winter2026_DouglasCollege/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="104" documentId="8_{08655895-4010-492B-B73A-F5D36A9F8AF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B371C32D-278F-4B5E-8FE8-78F7DCF23A27}"/>
+  <xr:revisionPtr revIDLastSave="135" documentId="8_{08655895-4010-492B-B73A-F5D36A9F8AF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0F0C5E6B-2E78-41F0-8095-29D68DBF36E4}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="794" uniqueCount="381">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="925" uniqueCount="413">
   <si>
     <t>CSIS 4495 - Applied Research Project</t>
   </si>
@@ -1178,6 +1178,102 @@
   </si>
   <si>
     <t>Mid-term Video Demonstration</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   3E: Multi-Turn Chatbot Enhancement</t>
+  </si>
+  <si>
+    <t>2026-02-25</t>
+  </si>
+  <si>
+    <t>Sprint 3</t>
+  </si>
+  <si>
+    <t>2026-02-26</t>
+  </si>
+  <si>
+    <t>2026-02-27</t>
+  </si>
+  <si>
+    <t>2026-02-28</t>
+  </si>
+  <si>
+    <t>2026-03-01</t>
+  </si>
+  <si>
+    <t>2026-03-02</t>
+  </si>
+  <si>
+    <t>Post-cruise return: Reviewed Sprint 3 roadmap tracker, organized project files and mockups into consolidated project workspace</t>
+  </si>
+  <si>
+    <t>Studied existing 1_Home.py placeholder code, compared against UI mockup, identified all sections needing rebuild</t>
+  </si>
+  <si>
+    <t>Rebuilt Home page Welcome Header section with personalized greeting using session_state username, added health overview subtitle</t>
+  </si>
+  <si>
+    <t>Created Quick Actions row (3 styled cards with icons: Check Symptoms, Find Facility, Health Info) with st.page_link() navigation</t>
+  </si>
+  <si>
+    <t>Created My Health Summary card querying SQLite database via get_assessment_stats() - displays total assessments, last check relative time, most common symptom with percentage</t>
+  </si>
+  <si>
+    <t>Created Recent Activity list showing 3 most recent assessments from database with color-coded urgency dots (green/yellow/red)</t>
+  </si>
+  <si>
+    <t>Added BC Health Tip of the Day banner with rotating BC-specific health tips and Find Nearest Pharmacy navigation button</t>
+  </si>
+  <si>
+    <t>Added most_common_symptom_count to get_assessment_stats() in database.py for percentage calculation (backward-compatible change)</t>
+  </si>
+  <si>
+    <t>Verified all dashboard data against SQLite database using Python queries - confirmed 33 assessments, Chest pain 33%, recent activity entries all match live data</t>
+  </si>
+  <si>
+    <t>Git commit - 'Sprint 3A: Rebuild Home Dashboard to match UI mockup'</t>
+  </si>
+  <si>
+    <t>Studied My Personal Health Dashboard mockup (2 pages), identified 5 sections: stat cards, trend chart, symptoms breakdown, assessment history table, date filter</t>
+  </si>
+  <si>
+    <t>Built dashboard layout with 4 stat summary cards (Total Checks, This Month, Most Common, Avg Urgency) with colored icon boxes and status indicators</t>
+  </si>
+  <si>
+    <t>Created Plotly filled area chart for Symptom Trends Over Time - grouped assessments by month, teal color scheme, responsive layout with export_plotly_chart()</t>
+  </si>
+  <si>
+    <t>Created Plotly donut pie chart for Symptoms Breakdown - shows distribution of primary symptoms with percentages, rare symptoms grouped as Other</t>
+  </si>
+  <si>
+    <t>Created Assessment History HTML table with styled colored badges (green Home Care, yellow Walk-in Clinic, orange Urgent Care, red Emergency)</t>
+  </si>
+  <si>
+    <t>Implemented date filter dropdown (All Time, Last 6 Months, Last 3 Months, Last Year) that filters all dashboard sections simultaneously</t>
+  </si>
+  <si>
+    <t>Fixed UI issues - Plotly X-axis tick intervals (dtick=5), donut chart label clipping (moved labels inside slices with legend below), button styling for Export Report and New Assessment</t>
+  </si>
+  <si>
+    <t>Automated data verification against SQLite - confirmed all 4 stat cards, trend chart, donut chart percentages, and history table entries match real database values</t>
+  </si>
+  <si>
+    <t>Git commit - 'Sprint 3B: Rebuild My Dashboard with Plotly charts, date filter, and live data'</t>
+  </si>
+  <si>
+    <t>Added auto-redirect in app.py to route users to Home Dashboard after login instead of showing old placeholder page; Git commit</t>
+  </si>
+  <si>
+    <t>Researched agentic AI frameworks in healthcare triage (reviewed Thamma 2025, Wang et al. 2024); Evaluated feasibility for project integration</t>
+  </si>
+  <si>
+    <t>Updated work log, prepared Progress Report 2, updated task tracker with Sprint 3A and 3B completion status</t>
+  </si>
+  <si>
+    <t>3A</t>
+  </si>
+  <si>
+    <t>3B</t>
   </si>
 </sst>
 </file>
@@ -1185,7 +1281,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd;@"/>
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
   </numFmts>
   <fonts count="20" x14ac:knownFonts="1">
     <font>
@@ -1318,7 +1414,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="25">
+  <fills count="26">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1441,6 +1537,12 @@
         <fgColor rgb="FFD6E4F0"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="8">
     <border>
@@ -1547,7 +1649,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="104">
+  <cellXfs count="105">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1720,6 +1822,25 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -1740,7 +1861,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1748,23 +1868,8 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="4" fillId="25" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2248,43 +2353,43 @@
     <col min="2" max="2" width="8" customWidth="1"/>
     <col min="3" max="3" width="10" customWidth="1"/>
     <col min="4" max="4" width="8" customWidth="1"/>
-    <col min="5" max="5" width="27.21875" style="69" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="34.21875" style="69" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="10" style="20" customWidth="1"/>
     <col min="7" max="7" width="209.77734375" style="23" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="95" t="s">
+      <c r="A1" s="103" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="92"/>
-      <c r="C1" s="92"/>
-      <c r="D1" s="92"/>
-      <c r="E1" s="92"/>
-      <c r="F1" s="93"/>
-      <c r="G1" s="94"/>
+      <c r="B1" s="89"/>
+      <c r="C1" s="89"/>
+      <c r="D1" s="89"/>
+      <c r="E1" s="89"/>
+      <c r="F1" s="101"/>
+      <c r="G1" s="102"/>
     </row>
     <row r="2" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="91" t="s">
+      <c r="A2" s="100" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="92"/>
-      <c r="C2" s="92"/>
-      <c r="D2" s="92"/>
-      <c r="E2" s="92"/>
-      <c r="F2" s="93"/>
-      <c r="G2" s="94"/>
+      <c r="B2" s="89"/>
+      <c r="C2" s="89"/>
+      <c r="D2" s="89"/>
+      <c r="E2" s="89"/>
+      <c r="F2" s="101"/>
+      <c r="G2" s="102"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3" s="87" t="s">
+      <c r="A3" s="96" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="88"/>
-      <c r="C3" s="88"/>
-      <c r="D3" s="88"/>
-      <c r="E3" s="88"/>
-      <c r="F3" s="89"/>
-      <c r="G3" s="90"/>
+      <c r="B3" s="97"/>
+      <c r="C3" s="97"/>
+      <c r="D3" s="97"/>
+      <c r="E3" s="97"/>
+      <c r="F3" s="98"/>
+      <c r="G3" s="99"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="F4" s="17"/>
@@ -4886,7 +4991,7 @@
       </c>
     </row>
     <row r="119" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A119" s="100">
+      <c r="A119" s="84">
         <v>46066</v>
       </c>
       <c r="B119" s="24" t="s">
@@ -4895,19 +5000,19 @@
       <c r="C119" s="1" t="s">
         <v>378</v>
       </c>
-      <c r="D119" s="101">
+      <c r="D119" s="85">
         <v>4</v>
       </c>
       <c r="E119" s="83" t="s">
-        <v>211</v>
-      </c>
-      <c r="F119" s="103"/>
+        <v>37</v>
+      </c>
+      <c r="F119" s="87"/>
       <c r="G119" s="21" t="s">
         <v>379</v>
       </c>
     </row>
     <row r="120" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A120" s="100">
+      <c r="A120" s="84">
         <v>46066</v>
       </c>
       <c r="B120" s="24" t="s">
@@ -4916,214 +5021,518 @@
       <c r="C120" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D120" s="102">
+      <c r="D120" s="86">
         <v>2</v>
       </c>
       <c r="E120" s="83" t="s">
-        <v>211</v>
-      </c>
-      <c r="F120" s="103"/>
+        <v>37</v>
+      </c>
+      <c r="F120" s="87"/>
       <c r="G120" s="21" t="s">
         <v>380</v>
       </c>
     </row>
     <row r="121" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A121" s="1"/>
-      <c r="B121" s="1"/>
-      <c r="C121" s="1"/>
-      <c r="D121" s="2"/>
-      <c r="E121" s="27"/>
-      <c r="F121" s="18"/>
-      <c r="G121" s="21"/>
+      <c r="A121" s="84" t="s">
+        <v>382</v>
+      </c>
+      <c r="B121" s="24" t="s">
+        <v>383</v>
+      </c>
+      <c r="C121" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D121" s="86">
+        <v>1</v>
+      </c>
+      <c r="E121" s="27" t="s">
+        <v>212</v>
+      </c>
+      <c r="F121" s="18" t="s">
+        <v>411</v>
+      </c>
+      <c r="G121" t="s">
+        <v>389</v>
+      </c>
     </row>
     <row r="122" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A122" s="1"/>
-      <c r="B122" s="1"/>
-      <c r="C122" s="1"/>
-      <c r="D122" s="2"/>
-      <c r="E122" s="25"/>
-      <c r="F122" s="18"/>
-      <c r="G122" s="21"/>
+      <c r="A122" s="84" t="s">
+        <v>382</v>
+      </c>
+      <c r="B122" s="24" t="s">
+        <v>383</v>
+      </c>
+      <c r="C122" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D122" s="86">
+        <v>0.5</v>
+      </c>
+      <c r="E122" s="27" t="s">
+        <v>212</v>
+      </c>
+      <c r="F122" s="18" t="s">
+        <v>411</v>
+      </c>
+      <c r="G122" t="s">
+        <v>390</v>
+      </c>
     </row>
     <row r="123" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A123" s="1"/>
-      <c r="B123" s="1"/>
-      <c r="C123" s="1"/>
-      <c r="D123" s="2"/>
-      <c r="E123" s="25"/>
-      <c r="F123" s="18"/>
-      <c r="G123" s="21"/>
+      <c r="A123" s="84" t="s">
+        <v>382</v>
+      </c>
+      <c r="B123" s="24" t="s">
+        <v>383</v>
+      </c>
+      <c r="C123" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D123" s="86">
+        <v>1</v>
+      </c>
+      <c r="E123" s="27" t="s">
+        <v>212</v>
+      </c>
+      <c r="F123" s="18" t="s">
+        <v>411</v>
+      </c>
+      <c r="G123" t="s">
+        <v>391</v>
+      </c>
     </row>
     <row r="124" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A124" s="1"/>
-      <c r="B124" s="1"/>
-      <c r="C124" s="1"/>
-      <c r="D124" s="2"/>
-      <c r="E124" s="25"/>
-      <c r="F124" s="18"/>
-      <c r="G124" s="21"/>
+      <c r="A124" s="84" t="s">
+        <v>384</v>
+      </c>
+      <c r="B124" s="24" t="s">
+        <v>383</v>
+      </c>
+      <c r="C124" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="D124" s="86">
+        <v>0.75</v>
+      </c>
+      <c r="E124" s="27" t="s">
+        <v>212</v>
+      </c>
+      <c r="F124" s="18" t="s">
+        <v>411</v>
+      </c>
+      <c r="G124" t="s">
+        <v>392</v>
+      </c>
     </row>
     <row r="125" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A125" s="1"/>
-      <c r="B125" s="1"/>
-      <c r="C125" s="1"/>
-      <c r="D125" s="2"/>
-      <c r="E125" s="25"/>
-      <c r="F125" s="18"/>
-      <c r="G125" s="21"/>
+      <c r="A125" s="84" t="s">
+        <v>384</v>
+      </c>
+      <c r="B125" s="24" t="s">
+        <v>383</v>
+      </c>
+      <c r="C125" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D125" s="86">
+        <v>1</v>
+      </c>
+      <c r="E125" s="27" t="s">
+        <v>212</v>
+      </c>
+      <c r="F125" s="18" t="s">
+        <v>411</v>
+      </c>
+      <c r="G125" t="s">
+        <v>393</v>
+      </c>
     </row>
     <row r="126" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A126" s="1"/>
-      <c r="B126" s="1"/>
-      <c r="C126" s="1"/>
-      <c r="D126" s="2"/>
-      <c r="E126" s="25"/>
-      <c r="F126" s="18"/>
-      <c r="G126" s="21"/>
+      <c r="A126" s="84" t="s">
+        <v>384</v>
+      </c>
+      <c r="B126" s="24" t="s">
+        <v>383</v>
+      </c>
+      <c r="C126" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="D126" s="86">
+        <v>0.75</v>
+      </c>
+      <c r="E126" s="27" t="s">
+        <v>212</v>
+      </c>
+      <c r="F126" s="18" t="s">
+        <v>411</v>
+      </c>
+      <c r="G126" t="s">
+        <v>394</v>
+      </c>
     </row>
     <row r="127" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A127" s="1"/>
-      <c r="B127" s="1"/>
-      <c r="C127" s="1"/>
-      <c r="D127" s="2"/>
-      <c r="E127" s="25"/>
-      <c r="F127" s="18"/>
-      <c r="G127" s="21"/>
+      <c r="A127" s="84" t="s">
+        <v>385</v>
+      </c>
+      <c r="B127" s="24" t="s">
+        <v>383</v>
+      </c>
+      <c r="C127" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D127" s="86">
+        <v>0.5</v>
+      </c>
+      <c r="E127" s="27" t="s">
+        <v>212</v>
+      </c>
+      <c r="F127" s="18" t="s">
+        <v>411</v>
+      </c>
+      <c r="G127" t="s">
+        <v>395</v>
+      </c>
     </row>
     <row r="128" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A128" s="1"/>
-      <c r="B128" s="1"/>
-      <c r="C128" s="1"/>
-      <c r="D128" s="2"/>
-      <c r="E128" s="25"/>
-      <c r="F128" s="18"/>
-      <c r="G128" s="21"/>
+      <c r="A128" s="84" t="s">
+        <v>385</v>
+      </c>
+      <c r="B128" s="24" t="s">
+        <v>383</v>
+      </c>
+      <c r="C128" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D128" s="86">
+        <v>0.5</v>
+      </c>
+      <c r="E128" s="27" t="s">
+        <v>212</v>
+      </c>
+      <c r="F128" s="18" t="s">
+        <v>411</v>
+      </c>
+      <c r="G128" t="s">
+        <v>396</v>
+      </c>
     </row>
     <row r="129" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A129" s="1"/>
-      <c r="B129" s="1"/>
-      <c r="C129" s="1"/>
-      <c r="D129" s="2"/>
-      <c r="E129" s="25"/>
-      <c r="F129" s="18"/>
-      <c r="G129" s="21"/>
+      <c r="A129" s="84" t="s">
+        <v>385</v>
+      </c>
+      <c r="B129" s="24" t="s">
+        <v>383</v>
+      </c>
+      <c r="C129" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D129" s="86">
+        <v>0.5</v>
+      </c>
+      <c r="E129" s="27" t="s">
+        <v>212</v>
+      </c>
+      <c r="F129" s="18" t="s">
+        <v>411</v>
+      </c>
+      <c r="G129" t="s">
+        <v>397</v>
+      </c>
     </row>
     <row r="130" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A130" s="1"/>
-      <c r="B130" s="1"/>
-      <c r="C130" s="1"/>
-      <c r="D130" s="2"/>
-      <c r="E130" s="25"/>
-      <c r="F130" s="18"/>
-      <c r="G130" s="21"/>
+      <c r="A130" s="84" t="s">
+        <v>385</v>
+      </c>
+      <c r="B130" s="24" t="s">
+        <v>383</v>
+      </c>
+      <c r="C130" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D130" s="86">
+        <v>0.25</v>
+      </c>
+      <c r="E130" s="27" t="s">
+        <v>212</v>
+      </c>
+      <c r="F130" s="18" t="s">
+        <v>411</v>
+      </c>
+      <c r="G130" t="s">
+        <v>398</v>
+      </c>
     </row>
     <row r="131" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A131" s="1"/>
-      <c r="B131" s="1"/>
-      <c r="C131" s="1"/>
-      <c r="D131" s="2"/>
-      <c r="E131" s="25"/>
-      <c r="F131" s="18"/>
-      <c r="G131" s="21"/>
+      <c r="A131" s="84" t="s">
+        <v>386</v>
+      </c>
+      <c r="B131" s="24" t="s">
+        <v>383</v>
+      </c>
+      <c r="C131" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D131" s="86">
+        <v>0.5</v>
+      </c>
+      <c r="E131" s="104" t="s">
+        <v>234</v>
+      </c>
+      <c r="F131" s="18" t="s">
+        <v>412</v>
+      </c>
+      <c r="G131" t="s">
+        <v>399</v>
+      </c>
     </row>
     <row r="132" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A132" s="1"/>
-      <c r="B132" s="1"/>
-      <c r="C132" s="1"/>
-      <c r="D132" s="2"/>
-      <c r="E132" s="25"/>
-      <c r="F132" s="18"/>
-      <c r="G132" s="21"/>
+      <c r="A132" s="84" t="s">
+        <v>386</v>
+      </c>
+      <c r="B132" s="24" t="s">
+        <v>383</v>
+      </c>
+      <c r="C132" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D132" s="86">
+        <v>1.5</v>
+      </c>
+      <c r="E132" s="104" t="s">
+        <v>234</v>
+      </c>
+      <c r="F132" s="18" t="s">
+        <v>412</v>
+      </c>
+      <c r="G132" t="s">
+        <v>400</v>
+      </c>
     </row>
     <row r="133" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A133" s="1"/>
-      <c r="B133" s="1"/>
-      <c r="C133" s="1"/>
-      <c r="D133" s="2"/>
-      <c r="E133" s="25"/>
-      <c r="F133" s="18"/>
-      <c r="G133" s="21"/>
+      <c r="A133" s="84" t="s">
+        <v>387</v>
+      </c>
+      <c r="B133" s="24" t="s">
+        <v>383</v>
+      </c>
+      <c r="C133" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D133" s="86">
+        <v>1.5</v>
+      </c>
+      <c r="E133" s="104" t="s">
+        <v>234</v>
+      </c>
+      <c r="F133" s="18" t="s">
+        <v>412</v>
+      </c>
+      <c r="G133" t="s">
+        <v>401</v>
+      </c>
     </row>
     <row r="134" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A134" s="1"/>
-      <c r="B134" s="1"/>
-      <c r="C134" s="1"/>
-      <c r="D134" s="2"/>
-      <c r="E134" s="25"/>
-      <c r="F134" s="18"/>
-      <c r="G134" s="21"/>
+      <c r="A134" s="84" t="s">
+        <v>387</v>
+      </c>
+      <c r="B134" s="24" t="s">
+        <v>383</v>
+      </c>
+      <c r="C134" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D134" s="86">
+        <v>1</v>
+      </c>
+      <c r="E134" s="104" t="s">
+        <v>234</v>
+      </c>
+      <c r="F134" s="18" t="s">
+        <v>412</v>
+      </c>
+      <c r="G134" t="s">
+        <v>402</v>
+      </c>
     </row>
     <row r="135" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A135" s="1"/>
-      <c r="B135" s="1"/>
-      <c r="C135" s="1"/>
-      <c r="D135" s="2"/>
-      <c r="E135" s="25"/>
-      <c r="F135" s="18"/>
-      <c r="G135" s="21"/>
+      <c r="A135" s="84" t="s">
+        <v>387</v>
+      </c>
+      <c r="B135" s="24" t="s">
+        <v>383</v>
+      </c>
+      <c r="C135" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D135" s="86">
+        <v>1</v>
+      </c>
+      <c r="E135" s="104" t="s">
+        <v>234</v>
+      </c>
+      <c r="F135" s="18" t="s">
+        <v>412</v>
+      </c>
+      <c r="G135" t="s">
+        <v>403</v>
+      </c>
     </row>
     <row r="136" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A136" s="1"/>
-      <c r="B136" s="1"/>
-      <c r="C136" s="1"/>
-      <c r="D136" s="2"/>
-      <c r="E136" s="25"/>
-      <c r="F136" s="18"/>
-      <c r="G136" s="21"/>
+      <c r="A136" s="84" t="s">
+        <v>388</v>
+      </c>
+      <c r="B136" s="24" t="s">
+        <v>383</v>
+      </c>
+      <c r="C136" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="D136" s="86">
+        <v>0.75</v>
+      </c>
+      <c r="E136" s="104" t="s">
+        <v>234</v>
+      </c>
+      <c r="F136" s="18" t="s">
+        <v>412</v>
+      </c>
+      <c r="G136" t="s">
+        <v>404</v>
+      </c>
     </row>
     <row r="137" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A137" s="1"/>
-      <c r="B137" s="1"/>
-      <c r="C137" s="1"/>
-      <c r="D137" s="2"/>
-      <c r="E137" s="25"/>
-      <c r="F137" s="18"/>
-      <c r="G137" s="21"/>
+      <c r="A137" s="84" t="s">
+        <v>388</v>
+      </c>
+      <c r="B137" s="24" t="s">
+        <v>383</v>
+      </c>
+      <c r="C137" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="D137" s="86">
+        <v>0.75</v>
+      </c>
+      <c r="E137" s="104" t="s">
+        <v>234</v>
+      </c>
+      <c r="F137" s="18" t="s">
+        <v>412</v>
+      </c>
+      <c r="G137" t="s">
+        <v>405</v>
+      </c>
     </row>
     <row r="138" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A138" s="1"/>
-      <c r="B138" s="1"/>
-      <c r="C138" s="1"/>
-      <c r="D138" s="2"/>
-      <c r="E138" s="25"/>
-      <c r="F138" s="18"/>
-      <c r="G138" s="21"/>
+      <c r="A138" s="84" t="s">
+        <v>388</v>
+      </c>
+      <c r="B138" s="24" t="s">
+        <v>383</v>
+      </c>
+      <c r="C138" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D138" s="86">
+        <v>0.5</v>
+      </c>
+      <c r="E138" s="104" t="s">
+        <v>234</v>
+      </c>
+      <c r="F138" s="18" t="s">
+        <v>412</v>
+      </c>
+      <c r="G138" t="s">
+        <v>406</v>
+      </c>
     </row>
     <row r="139" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A139" s="1"/>
-      <c r="B139" s="1"/>
-      <c r="C139" s="1"/>
-      <c r="D139" s="2"/>
-      <c r="E139" s="25"/>
-      <c r="F139" s="18"/>
-      <c r="G139" s="21"/>
+      <c r="A139" s="84" t="s">
+        <v>388</v>
+      </c>
+      <c r="B139" s="24" t="s">
+        <v>383</v>
+      </c>
+      <c r="C139" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D139" s="86">
+        <v>0.25</v>
+      </c>
+      <c r="E139" s="104" t="s">
+        <v>234</v>
+      </c>
+      <c r="F139" s="18" t="s">
+        <v>412</v>
+      </c>
+      <c r="G139" t="s">
+        <v>407</v>
+      </c>
     </row>
     <row r="140" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A140" s="1"/>
-      <c r="B140" s="1"/>
-      <c r="C140" s="1"/>
-      <c r="D140" s="2"/>
-      <c r="E140" s="25"/>
-      <c r="F140" s="18"/>
-      <c r="G140" s="21"/>
+      <c r="A140" s="84" t="s">
+        <v>388</v>
+      </c>
+      <c r="B140" s="24" t="s">
+        <v>383</v>
+      </c>
+      <c r="C140" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D140" s="86">
+        <v>0.25</v>
+      </c>
+      <c r="E140" s="104" t="s">
+        <v>234</v>
+      </c>
+      <c r="F140" s="18" t="s">
+        <v>412</v>
+      </c>
+      <c r="G140" t="s">
+        <v>408</v>
+      </c>
     </row>
     <row r="141" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A141" s="1"/>
-      <c r="B141" s="1"/>
-      <c r="C141" s="1"/>
-      <c r="D141" s="2"/>
-      <c r="E141" s="25"/>
+      <c r="A141" s="84" t="s">
+        <v>388</v>
+      </c>
+      <c r="B141" s="24" t="s">
+        <v>383</v>
+      </c>
+      <c r="C141" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="D141" s="86">
+        <v>0.75</v>
+      </c>
+      <c r="E141" s="25" t="s">
+        <v>17</v>
+      </c>
       <c r="F141" s="18"/>
-      <c r="G141" s="21"/>
+      <c r="G141" t="s">
+        <v>409</v>
+      </c>
     </row>
     <row r="142" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A142" s="1"/>
-      <c r="B142" s="1"/>
-      <c r="C142" s="1"/>
-      <c r="D142" s="2"/>
-      <c r="E142" s="25"/>
+      <c r="A142" s="84" t="s">
+        <v>388</v>
+      </c>
+      <c r="B142" s="24" t="s">
+        <v>383</v>
+      </c>
+      <c r="C142" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="D142" s="86">
+        <v>0.75</v>
+      </c>
+      <c r="E142" s="25" t="s">
+        <v>37</v>
+      </c>
       <c r="F142" s="18"/>
-      <c r="G142" s="21"/>
+      <c r="G142" t="s">
+        <v>410</v>
+      </c>
     </row>
     <row r="143" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A143" s="1"/>
@@ -5171,15 +5580,15 @@
       <c r="G147" s="21"/>
     </row>
     <row r="148" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A148" s="84" t="s">
+      <c r="A148" s="93" t="s">
         <v>137</v>
       </c>
-      <c r="B148" s="85"/>
-      <c r="C148" s="85"/>
-      <c r="D148" s="86"/>
+      <c r="B148" s="94"/>
+      <c r="C148" s="94"/>
+      <c r="D148" s="95"/>
       <c r="E148" s="74">
         <f>SUM(D6:D147)</f>
-        <v>85.6</v>
+        <v>101.85</v>
       </c>
       <c r="F148" s="19"/>
       <c r="G148" s="22"/>
@@ -5274,7 +5683,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:N66"/>
+  <dimension ref="A1:N67"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="35" customWidth="1"/>
@@ -5282,31 +5691,31 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="22.8" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="99" t="s">
+      <c r="A1" s="92" t="s">
         <v>138</v>
       </c>
-      <c r="B1" s="92"/>
-      <c r="C1" s="92"/>
-      <c r="D1" s="92"/>
-      <c r="E1" s="92"/>
-      <c r="F1" s="92"/>
-      <c r="G1" s="92"/>
-      <c r="H1" s="92"/>
-      <c r="I1" s="92"/>
-      <c r="J1" s="92"/>
-      <c r="K1" s="92"/>
-      <c r="L1" s="92"/>
-      <c r="M1" s="92"/>
-      <c r="N1" s="92"/>
+      <c r="B1" s="89"/>
+      <c r="C1" s="89"/>
+      <c r="D1" s="89"/>
+      <c r="E1" s="89"/>
+      <c r="F1" s="89"/>
+      <c r="G1" s="89"/>
+      <c r="H1" s="89"/>
+      <c r="I1" s="89"/>
+      <c r="J1" s="89"/>
+      <c r="K1" s="89"/>
+      <c r="L1" s="89"/>
+      <c r="M1" s="89"/>
+      <c r="N1" s="89"/>
     </row>
     <row r="3" spans="1:14" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="96" t="s">
+      <c r="A3" s="88" t="s">
         <v>139</v>
       </c>
-      <c r="B3" s="92"/>
-      <c r="C3" s="92"/>
-      <c r="D3" s="92"/>
-      <c r="E3" s="92"/>
+      <c r="B3" s="89"/>
+      <c r="C3" s="89"/>
+      <c r="D3" s="89"/>
+      <c r="E3" s="89"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4" s="34" t="s">
@@ -5336,7 +5745,7 @@
         <v>5</v>
       </c>
       <c r="D5" s="38">
-        <f>B45</f>
+        <f>B46</f>
         <v>11.85</v>
       </c>
       <c r="E5" s="39">
@@ -5355,7 +5764,7 @@
         <v>15</v>
       </c>
       <c r="D6" s="38">
-        <f>SUM(B46:B50)</f>
+        <f>SUM(B47:B51)</f>
         <v>14.26</v>
       </c>
       <c r="E6" s="39">
@@ -5374,8 +5783,8 @@
         <v>25</v>
       </c>
       <c r="D7" s="38">
-        <f>SUM(B51:B54)</f>
-        <v>35.99</v>
+        <f>SUM(B52:B55)</f>
+        <v>29.990000000000002</v>
       </c>
       <c r="E7" s="39">
         <f t="shared" si="0"/>
@@ -5393,12 +5802,12 @@
         <v>20</v>
       </c>
       <c r="D8" s="38">
-        <f>SUM(B55:B58)</f>
-        <v>0</v>
+        <f>SUM(B56:B59)</f>
+        <v>6.75</v>
       </c>
       <c r="E8" s="39">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.33750000000000002</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.3">
@@ -5412,7 +5821,7 @@
         <v>20</v>
       </c>
       <c r="D9" s="38">
-        <f>SUM(B59:B60)</f>
+        <f>SUM(B60:B61)</f>
         <v>0</v>
       </c>
       <c r="E9" s="39">
@@ -5431,7 +5840,7 @@
         <v>15</v>
       </c>
       <c r="D10" s="38">
-        <f>SUM(B61:B62)</f>
+        <f>SUM(B62:B63)</f>
         <v>0</v>
       </c>
       <c r="E10" s="39">
@@ -5450,12 +5859,12 @@
         <v>18</v>
       </c>
       <c r="D11" s="38">
-        <f>SUM(B63)</f>
-        <v>6.5</v>
+        <f>SUM(B64)</f>
+        <v>13.25</v>
       </c>
       <c r="E11" s="39">
         <f t="shared" si="0"/>
-        <v>0.3611111111111111</v>
+        <v>0.73611111111111116</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.3">
@@ -5469,30 +5878,30 @@
       </c>
       <c r="D12" s="55">
         <f>SUM(D5:D11)</f>
-        <v>68.599999999999994</v>
+        <v>76.099999999999994</v>
       </c>
       <c r="E12" s="56">
         <f>IF(C12=0,0,D12/C12)</f>
-        <v>0.58135593220338977</v>
+        <v>0.64491525423728813</v>
       </c>
     </row>
     <row r="14" spans="1:14" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="97" t="s">
+      <c r="A14" s="90" t="s">
         <v>152</v>
       </c>
-      <c r="B14" s="98"/>
-      <c r="C14" s="98"/>
-      <c r="D14" s="98"/>
-      <c r="E14" s="98"/>
-      <c r="F14" s="98"/>
-      <c r="G14" s="98"/>
-      <c r="H14" s="98"/>
-      <c r="I14" s="98"/>
-      <c r="J14" s="98"/>
-      <c r="K14" s="98"/>
-      <c r="L14" s="98"/>
-      <c r="M14" s="98"/>
-      <c r="N14" s="98"/>
+      <c r="B14" s="91"/>
+      <c r="C14" s="91"/>
+      <c r="D14" s="91"/>
+      <c r="E14" s="91"/>
+      <c r="F14" s="91"/>
+      <c r="G14" s="91"/>
+      <c r="H14" s="91"/>
+      <c r="I14" s="91"/>
+      <c r="J14" s="91"/>
+      <c r="K14" s="91"/>
+      <c r="L14" s="91"/>
+      <c r="M14" s="91"/>
+      <c r="N14" s="91"/>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A15" s="34" t="s">
@@ -5887,8 +6296,8 @@
       <c r="N33" s="53"/>
     </row>
     <row r="34" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A34" s="52" t="s">
-        <v>197</v>
+      <c r="A34" s="81" t="s">
+        <v>381</v>
       </c>
       <c r="B34" s="53"/>
       <c r="C34" s="53"/>
@@ -5896,57 +6305,55 @@
       <c r="E34" s="53"/>
       <c r="F34" s="53"/>
       <c r="G34" s="53"/>
-      <c r="H34" s="47"/>
-      <c r="I34" s="47"/>
-      <c r="J34" s="47"/>
+      <c r="H34" s="45"/>
+      <c r="I34" s="53"/>
+      <c r="J34" s="63"/>
       <c r="K34" s="63"/>
       <c r="L34" s="53"/>
       <c r="M34" s="53"/>
       <c r="N34" s="53"/>
     </row>
     <row r="35" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A35" s="81" t="s">
-        <v>198</v>
+      <c r="A35" s="52" t="s">
+        <v>197</v>
       </c>
       <c r="B35" s="53"/>
       <c r="C35" s="53"/>
       <c r="D35" s="53"/>
       <c r="E35" s="53"/>
-      <c r="F35" s="64" t="s">
-        <v>199</v>
-      </c>
+      <c r="F35" s="53"/>
       <c r="G35" s="53"/>
       <c r="H35" s="47"/>
       <c r="I35" s="47"/>
-      <c r="J35" s="53"/>
-      <c r="K35" s="53"/>
+      <c r="J35" s="47"/>
+      <c r="K35" s="63"/>
       <c r="L35" s="53"/>
       <c r="M35" s="53"/>
       <c r="N35" s="53"/>
     </row>
     <row r="36" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A36" s="81" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="B36" s="53"/>
       <c r="C36" s="53"/>
       <c r="D36" s="53"/>
       <c r="E36" s="53"/>
-      <c r="F36" s="53"/>
+      <c r="F36" s="64" t="s">
+        <v>199</v>
+      </c>
       <c r="G36" s="53"/>
-      <c r="H36" s="53"/>
+      <c r="H36" s="47"/>
       <c r="I36" s="47"/>
-      <c r="J36" s="47"/>
+      <c r="J36" s="53"/>
       <c r="K36" s="53"/>
       <c r="L36" s="53"/>
       <c r="M36" s="53"/>
-      <c r="N36" s="64" t="s">
-        <v>199</v>
-      </c>
+      <c r="N36" s="53"/>
     </row>
     <row r="37" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A37" s="52" t="s">
-        <v>201</v>
+      <c r="A37" s="81" t="s">
+        <v>200</v>
       </c>
       <c r="B37" s="53"/>
       <c r="C37" s="53"/>
@@ -5955,16 +6362,18 @@
       <c r="F37" s="53"/>
       <c r="G37" s="53"/>
       <c r="H37" s="53"/>
-      <c r="I37" s="53"/>
-      <c r="J37" s="49"/>
-      <c r="K37" s="49"/>
-      <c r="L37" s="49"/>
+      <c r="I37" s="47"/>
+      <c r="J37" s="47"/>
+      <c r="K37" s="53"/>
+      <c r="L37" s="53"/>
       <c r="M37" s="53"/>
-      <c r="N37" s="53"/>
+      <c r="N37" s="64" t="s">
+        <v>199</v>
+      </c>
     </row>
     <row r="38" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A38" s="81" t="s">
-        <v>202</v>
+      <c r="A38" s="52" t="s">
+        <v>201</v>
       </c>
       <c r="B38" s="53"/>
       <c r="C38" s="53"/>
@@ -5976,13 +6385,13 @@
       <c r="I38" s="53"/>
       <c r="J38" s="49"/>
       <c r="K38" s="49"/>
-      <c r="L38" s="53"/>
+      <c r="L38" s="49"/>
       <c r="M38" s="53"/>
       <c r="N38" s="53"/>
     </row>
     <row r="39" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A39" s="81" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B39" s="53"/>
       <c r="C39" s="53"/>
@@ -5992,15 +6401,15 @@
       <c r="G39" s="53"/>
       <c r="H39" s="53"/>
       <c r="I39" s="53"/>
-      <c r="J39" s="53"/>
+      <c r="J39" s="49"/>
       <c r="K39" s="49"/>
-      <c r="L39" s="49"/>
+      <c r="L39" s="53"/>
       <c r="M39" s="53"/>
       <c r="N39" s="53"/>
     </row>
-    <row r="40" spans="1:14" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="52" t="s">
-        <v>204</v>
+    <row r="40" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A40" s="81" t="s">
+        <v>203</v>
       </c>
       <c r="B40" s="53"/>
       <c r="C40" s="53"/>
@@ -6011,251 +6420,269 @@
       <c r="H40" s="53"/>
       <c r="I40" s="53"/>
       <c r="J40" s="53"/>
-      <c r="K40" s="53"/>
-      <c r="L40" s="51"/>
-      <c r="M40" s="51"/>
-      <c r="N40" s="51"/>
+      <c r="K40" s="49"/>
+      <c r="L40" s="49"/>
+      <c r="M40" s="53"/>
+      <c r="N40" s="53"/>
     </row>
     <row r="41" spans="1:14" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="80"/>
-    </row>
-    <row r="42" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A42" s="3" t="s">
+      <c r="A41" s="52" t="s">
+        <v>204</v>
+      </c>
+      <c r="B41" s="53"/>
+      <c r="C41" s="53"/>
+      <c r="D41" s="53"/>
+      <c r="E41" s="53"/>
+      <c r="F41" s="53"/>
+      <c r="G41" s="53"/>
+      <c r="H41" s="53"/>
+      <c r="I41" s="53"/>
+      <c r="J41" s="53"/>
+      <c r="K41" s="53"/>
+      <c r="L41" s="51"/>
+      <c r="M41" s="51"/>
+      <c r="N41" s="51"/>
+    </row>
+    <row r="42" spans="1:14" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="80"/>
+    </row>
+    <row r="43" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A43" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B42" s="3" t="s">
+      <c r="B43" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C42" s="75"/>
-    </row>
-    <row r="43" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A43" s="65" t="s">
+      <c r="C43" s="75"/>
+    </row>
+    <row r="44" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A44" s="65" t="s">
         <v>205</v>
       </c>
-      <c r="B43" s="5"/>
-      <c r="C43" s="4"/>
-    </row>
-    <row r="44" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A44" s="34" t="s">
+      <c r="B44" s="5"/>
+      <c r="C44" s="4"/>
+    </row>
+    <row r="45" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A45" s="34" t="s">
         <v>7</v>
       </c>
-      <c r="B44" s="66" t="s">
+      <c r="B45" s="66" t="s">
         <v>6</v>
       </c>
-      <c r="C44" s="4"/>
-    </row>
-    <row r="45" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A45" s="36" t="s">
+      <c r="C45" s="4"/>
+    </row>
+    <row r="46" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A46" s="36" t="s">
         <v>12</v>
       </c>
-      <c r="B45" s="38">
+      <c r="B46" s="38">
         <f>SUMIF('Work Log'!E:E,"0: Environment Setup",'Work Log'!D:D)</f>
         <v>11.85</v>
       </c>
-      <c r="C45" s="4"/>
-    </row>
-    <row r="46" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A46" s="41" t="s">
+      <c r="C46" s="4"/>
+    </row>
+    <row r="47" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A47" s="41" t="s">
         <v>94</v>
       </c>
-      <c r="B46" s="38">
+      <c r="B47" s="38">
         <f>SUMIF('Work Log'!E:E,"1A: UI Mockups",'Work Log'!D:D)</f>
         <v>2.81</v>
       </c>
-      <c r="C46" s="4"/>
-    </row>
-    <row r="47" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A47" s="41" t="s">
+      <c r="C47" s="4"/>
+    </row>
+    <row r="48" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A48" s="41" t="s">
         <v>113</v>
       </c>
-      <c r="B47" s="38">
+      <c r="B48" s="38">
         <f>SUMIF('Work Log'!E:E,"1B: Project Structure",'Work Log'!D:D)</f>
         <v>0.67</v>
       </c>
-      <c r="C47" s="4"/>
-    </row>
-    <row r="48" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A48" s="41" t="s">
+      <c r="C48" s="4"/>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A49" s="41" t="s">
         <v>121</v>
       </c>
-      <c r="B48" s="38">
+      <c r="B49" s="38">
         <f>SUMIF('Work Log'!E:E,"1C: Database Setup",'Work Log'!D:D)</f>
         <v>3.18</v>
       </c>
-      <c r="C48" s="4"/>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A49" s="41" t="s">
+      <c r="C49" s="4"/>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A50" s="41" t="s">
         <v>206</v>
       </c>
-      <c r="B49" s="38">
+      <c r="B50" s="38">
         <f>SUMIF('Work Log'!E:E,"1D: Authentication Feature",'Work Log'!D:D)</f>
         <v>6</v>
       </c>
-      <c r="C49" s="4"/>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A50" s="41" t="s">
+      <c r="C50" s="4"/>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A51" s="41" t="s">
         <v>207</v>
       </c>
-      <c r="B50" s="38">
+      <c r="B51" s="38">
         <f>SUMIF('Work Log'!E:E,"1E: Basic Navigation",'Work Log'!D:D)</f>
         <v>1.5999999999999999</v>
       </c>
-      <c r="C50" s="4"/>
-    </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A51" s="43" t="s">
+      <c r="C51" s="4"/>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A52" s="43" t="s">
         <v>208</v>
       </c>
-      <c r="B51" s="38">
+      <c r="B52" s="38">
         <f>SUMIF('Work Log'!E:E,"2A: Open AI Integration",'Work Log'!D:D)</f>
         <v>2.08</v>
       </c>
-      <c r="C51" s="4"/>
-    </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A52" s="43" t="s">
+      <c r="C52" s="4"/>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A53" s="43" t="s">
         <v>209</v>
       </c>
-      <c r="B52" s="38">
+      <c r="B53" s="38">
         <f>SUMIF('Work Log'!E:E,"2B: Safety Layer - CTAS Rules",'Work Log'!D:D)</f>
         <v>2.75</v>
       </c>
-      <c r="C52" s="4"/>
-    </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A53" s="43" t="s">
+      <c r="C53" s="4"/>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A54" s="43" t="s">
         <v>210</v>
       </c>
-      <c r="B53" s="38">
+      <c r="B54" s="38">
         <f>SUMIF('Work Log'!E:E,"2C: ML Model Training",'Work Log'!D:D)</f>
         <v>9</v>
       </c>
-      <c r="C53" s="4"/>
-    </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A54" s="43" t="s">
+      <c r="C54" s="4"/>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A55" s="43" t="s">
         <v>211</v>
       </c>
-      <c r="B54" s="38">
+      <c r="B55" s="38">
         <f>SUMIF('Work Log'!E:E,"2D: Chatbot UI + Integration",'Work Log'!D:D)</f>
-        <v>22.16</v>
-      </c>
-      <c r="C54" s="4"/>
-    </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A55" s="45" t="s">
-        <v>212</v>
-      </c>
-      <c r="B55" s="38">
-        <f>SUMIF('Work Log'!E:E,"3A: Home Dashboard",'Work Log'!D:D)</f>
-        <v>0</v>
+        <v>16.16</v>
       </c>
       <c r="C55" s="4"/>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A56" s="45" t="s">
+        <v>212</v>
+      </c>
+      <c r="B56" s="38">
+        <f>SUMIF('Work Log'!E:E,"3A: Home Dashboard",'Work Log'!D:D)</f>
+        <v>6.75</v>
+      </c>
+      <c r="C56" s="4"/>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A57" s="45" t="s">
         <v>213</v>
       </c>
-      <c r="B56" s="38">
+      <c r="B57" s="38">
         <f>SUMIF('Work Log'!E:E,"3B: My Dashboard - Personal Analytics",'Work Log'!D:D)</f>
         <v>0</v>
       </c>
-      <c r="C56" s="4"/>
-    </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A57" s="45" t="s">
+      <c r="C57" s="4"/>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A58" s="45" t="s">
         <v>214</v>
       </c>
-      <c r="B57" s="38">
+      <c r="B58" s="38">
         <f>SUMIF('Work Log'!E:E,"3C: Facility Finder",'Work Log'!D:D)</f>
         <v>0</v>
       </c>
-      <c r="C57" s="4"/>
-    </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A58" s="45" t="s">
+      <c r="C58" s="4"/>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A59" s="45" t="s">
         <v>215</v>
       </c>
-      <c r="B58" s="38">
+      <c r="B59" s="38">
         <f>SUMIF('Work Log'!E:E,"3D: Health Education Library",'Work Log'!D:D)</f>
         <v>0</v>
       </c>
-      <c r="C58" s="4"/>
-    </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A59" s="47" t="s">
+      <c r="C59" s="4"/>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A60" s="47" t="s">
         <v>216</v>
       </c>
-      <c r="B59" s="38">
+      <c r="B60" s="38">
         <f>SUMIF('Work Log'!E:E,"4A: System Analytics Data",'Work Log'!D:D)</f>
         <v>0</v>
       </c>
-      <c r="C59" s="4"/>
-    </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A60" s="47" t="s">
+      <c r="C60" s="4"/>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A61" s="47" t="s">
         <v>217</v>
       </c>
-      <c r="B60" s="38">
+      <c r="B61" s="38">
         <f>SUMIF('Work Log'!E:E,"4B: System Analytics Dashboard",'Work Log'!D:D)</f>
         <v>0</v>
       </c>
-      <c r="C60" s="4"/>
-    </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A61" s="49" t="s">
+      <c r="C61" s="4"/>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A62" s="49" t="s">
         <v>218</v>
       </c>
-      <c r="B61" s="38">
+      <c r="B62" s="38">
         <f>SUMIF('Work Log'!E:E,"5A: Deployment",'Work Log'!D:D)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A62" s="49" t="s">
+    <row r="63" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A63" s="49" t="s">
         <v>219</v>
       </c>
-      <c r="B62" s="38">
+      <c r="B63" s="38">
         <f>SUMIF('Work Log'!E:E,"5B: Testing",'Work Log'!D:D)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A63" s="51" t="s">
+    <row r="64" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A64" s="51" t="s">
         <v>37</v>
       </c>
-      <c r="B63" s="38">
+      <c r="B64" s="38">
         <f>SUMIF('Work Log'!E:E,"6: Documentation + Submission",'Work Log'!D:D)</f>
-        <v>6.5</v>
-      </c>
-    </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A64" s="67" t="s">
+        <v>13.25</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A65" s="67" t="s">
         <v>17</v>
       </c>
-      <c r="B64" s="38">
+      <c r="B65" s="38">
         <f>SUMIF('Work Log'!E:E,"Learning &amp; Research",'Work Log'!D:D)</f>
-        <v>17</v>
-      </c>
-    </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A65" s="68" t="s">
+        <v>17.75</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A66" s="68" t="s">
         <v>220</v>
       </c>
-      <c r="B65" s="38">
+      <c r="B66" s="38">
         <f>SUMIF('Work Log'!E:E,"Proof of Concept",'Work Log'!D:D)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A66" s="52" t="s">
+    <row r="67" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A67" s="52" t="s">
         <v>151</v>
       </c>
-      <c r="B66" s="55">
-        <f>SUM(B45:B65)</f>
-        <v>85.600000000000009</v>
+      <c r="B67" s="55">
+        <f>SUM(B46:B66)</f>
+        <v>93.850000000000009</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Uploaded Progress Report 4 & Updated Excel Work Log (138.85 total hrs)
</commit_message>
<xml_diff>
--- a/DocumentsAndReports/worklog/WorkLog_DesmondChua_W26_4495_S2.xlsx
+++ b/DocumentsAndReports/worklog/WorkLog_DesmondChua_W26_4495_S2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d4f25ae689476683/Desmond_New/BC-Health-Platform/DocumentsAndReports/worklog/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="159" documentId="8_{08655895-4010-492B-B73A-F5D36A9F8AF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{47B02F83-99C8-4CB2-8FB6-80065E4D42CC}"/>
+  <xr:revisionPtr revIDLastSave="182" documentId="8_{08655895-4010-492B-B73A-F5D36A9F8AF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DBECE850-859A-40A1-B437-F926111F1D88}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1030" uniqueCount="440">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1129" uniqueCount="466">
   <si>
     <t>CSIS 4495 - Applied Research Project</t>
   </si>
@@ -1355,6 +1355,84 @@
   </si>
   <si>
     <t>Prepared Progress Report 3; updated commit history, work log entries, and Gantt chart for PR3 reporting period (Mar 3–9)</t>
+  </si>
+  <si>
+    <t>Sprint 3D Research: Reviewed HealthLinkBC content categories and identified 8 topic areas for the Health Library (Pain &amp; Injury, Cold &amp; Flu, Medications, Prevention &amp; Wellness, Mental Health, Heart Health, Child Health, Emergency Care)</t>
+  </si>
+  <si>
+    <t>Sprint 3D Research: Designed JSON schema for health_articles.json — identified required fields: id, title, category, summary, content, tags, read_time, source_url, banner_color; mapped 18 article topics across 8 categories</t>
+  </si>
+  <si>
+    <t>1 hr 15 min</t>
+  </si>
+  <si>
+    <t>Sprint 3D: Drafted prompt for Claude Code to generate health_articles.json with 18 BC-specific health articles and Health Library page with full page structure matching mockup; reviewed and committed first draft</t>
+  </si>
+  <si>
+    <t>Sprint 3D: Tested initial Health Library page — identified and documented UI bugs: duplicate category grid rendering, search section layout issues, incorrect section header styling; planned targeted fix approach</t>
+  </si>
+  <si>
+    <t>Sprint 3D Fix: Corrected Health Library UI — removed duplicate st.button() row above category icon cards, replaced teal section_header() on Browse by Category with plain st.markdown(), redesigned search card layout</t>
+  </si>
+  <si>
+    <t>Sprint 3D Fix: Resolved ghost input box appearing between page subtitle and search card — root cause identified as orphaned HTML div wrappers auto-closing before Streamlit widgets rendered; replaced with CSS :has() marker injection pattern</t>
+  </si>
+  <si>
+    <t>Sprint 3D: Implemented search logic — keyword filtering against article title, category, tags, and summary fields using session_state (hl_search_query); results grid with 3-column card layout, Clear Search button, no-results fallback message</t>
+  </si>
+  <si>
+    <t>Sprint 3D: Wired Browse by Category Select buttons to filter articles — hl_selected_category session state, 3-column filtered results grid, mutual exclusivity with search filter; tested all 8 categories</t>
+  </si>
+  <si>
+    <t>Sprint 3D: Verified Popular Topics section — 4 coloured banner cards (blue/green/purple/red), expandable full article content, Visit Source external links; confirmed all expanders and links functional</t>
+  </si>
+  <si>
+    <t>Sprint 3D: Implemented UX improvement — wrapped All Articles section in collapsed st.expander() to reduce cognitive overload from 18 article cards; applied teal CSS :has() styling to match platform section header design system</t>
+  </si>
+  <si>
+    <t>Sprint 3D: Standardized font weight across all teal section headers (700 weight, 16px, 0.01em letter-spacing); confirmed Official BC Health Resources section (HealthLinkBC, BCCDC, BC Health Services cards) rendering correctly</t>
+  </si>
+  <si>
+    <t>Sprint 3D: Final review and testing of complete Health Library — search, category filter, popular topics, all articles expander, BC health resources, footer disclaimer; committed all Sprint 3D work to GitHub</t>
+  </si>
+  <si>
+    <t>Sprint 4</t>
+  </si>
+  <si>
+    <t>Sprint 4A Research: Designed synthetic data model for System Analytics — defined 3 patient engagement tiers (Healthy/Occasional, Moderate Users, High-Frequency/Chronic) with realistic assessment frequency and urgency distributions; drafted data generation requirements</t>
+  </si>
+  <si>
+    <t>Sprint 4A: Developed generate_synthetic_data.py — 200 patients across 3 tiers, 5,000 assessment records with tier-weighted urgency distributions, flu season patterns (Nov–Feb spike), chronic symptom elevation for Tier 3; post-generation Emergency cap at ≤5%</t>
+  </si>
+  <si>
+    <t>Sprint 4A: Validated synthetic_assessments.csv output — confirmed 5,000 records, Emergency at exactly 5.0% (250 records), age distributions match tier specifications, top symptoms reflect chronic condition elevation for Tier 3 patients; committed to GitHub</t>
+  </si>
+  <si>
+    <t>Sprint 4B: Built System Analytics Dashboard page — page header with Export Report placeholder and date range filter dropdown (All Time default), CSV data loading with os.path relative resolution, @st.cache_data, 4 KPI cards with teal headers (Total Users, Active This Week, Total Assessments, Avg Assessment Time)</t>
+  </si>
+  <si>
+    <t>1 hr 45 min</t>
+  </si>
+  <si>
+    <t>Sprint 4B: Added 4 Plotly charts — horizontal bar chart (top 10 symptoms with clinical severity colour coding: red=Serious/Chronic, amber=Infectious, blue=General), Urgency Distribution donut, Usage by BC Health Authority donut (5 health authority regions mapped from cities), Assessment Trends line chart with numpy.polyfit orange trendline</t>
+  </si>
+  <si>
+    <t>Sprint 4B: Implemented K-Means unsupervised clustering — per-patient aggregation (age, assessment count, urgent ratio, chronic ratio), StandardScaler normalization, KMeans(n_clusters=3), automatic cluster naming by combined severity score; scatter plot visualization with bubble size = age; 3 cluster summary cards</t>
+  </si>
+  <si>
+    <t>Sprint 4B: Final verification and testing — date range filter wiring confirmed across all KPI cards and charts, K-Means cluster separation validated (Chronic/Elderly avg age 73, High-Risk avg age 47, Healthy/Occasional avg age 29); committed all Sprint 4A and 4B work to GitHub</t>
+  </si>
+  <si>
+    <t>3D</t>
+  </si>
+  <si>
+    <t>4A</t>
+  </si>
+  <si>
+    <t>4B</t>
+  </si>
+  <si>
+    <t>Prepared Progress Report 4; updated commit history, work log entries, and timeline for PR4 reporting period (Mar 10–16); added screenshots and submitted to Blackboard</t>
   </si>
 </sst>
 </file>
@@ -1918,6 +1996,25 @@
     <xf numFmtId="0" fontId="4" fillId="25" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -1950,25 +2047,6 @@
     <xf numFmtId="0" fontId="19" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -2155,6 +2233,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2442,7 +2524,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G165"/>
+  <dimension ref="A1:G185"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -2451,41 +2533,41 @@
     <col min="4" max="4" width="8" customWidth="1"/>
     <col min="5" max="5" width="34.21875" style="68" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="10" style="19" customWidth="1"/>
-    <col min="7" max="7" width="209.77734375" style="22" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="255.77734375" style="22" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="99" t="s">
+      <c r="A1" s="106" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="96"/>
-      <c r="C1" s="96"/>
-      <c r="D1" s="96"/>
-      <c r="E1" s="96"/>
-      <c r="F1" s="97"/>
-      <c r="G1" s="98"/>
+      <c r="B1" s="103"/>
+      <c r="C1" s="103"/>
+      <c r="D1" s="103"/>
+      <c r="E1" s="103"/>
+      <c r="F1" s="104"/>
+      <c r="G1" s="105"/>
     </row>
     <row r="2" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="95" t="s">
+      <c r="A2" s="102" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="96"/>
-      <c r="C2" s="96"/>
-      <c r="D2" s="96"/>
-      <c r="E2" s="96"/>
-      <c r="F2" s="97"/>
-      <c r="G2" s="98"/>
+      <c r="B2" s="103"/>
+      <c r="C2" s="103"/>
+      <c r="D2" s="103"/>
+      <c r="E2" s="103"/>
+      <c r="F2" s="104"/>
+      <c r="G2" s="105"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3" s="91" t="s">
+      <c r="A3" s="98" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="92"/>
-      <c r="C3" s="92"/>
-      <c r="D3" s="92"/>
-      <c r="E3" s="92"/>
-      <c r="F3" s="93"/>
-      <c r="G3" s="94"/>
+      <c r="B3" s="99"/>
+      <c r="C3" s="99"/>
+      <c r="D3" s="99"/>
+      <c r="E3" s="99"/>
+      <c r="F3" s="100"/>
+      <c r="G3" s="101"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="F4" s="16"/>
@@ -5631,7 +5713,7 @@
       </c>
     </row>
     <row r="143" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A143" s="105">
+      <c r="A143" s="89">
         <v>46084</v>
       </c>
       <c r="B143" s="23" t="s">
@@ -5640,7 +5722,7 @@
       <c r="C143" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="D143" s="108">
+      <c r="D143" s="92">
         <v>1</v>
       </c>
       <c r="E143" s="24" t="s">
@@ -5652,7 +5734,7 @@
       </c>
     </row>
     <row r="144" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A144" s="105">
+      <c r="A144" s="89">
         <v>46084</v>
       </c>
       <c r="B144" s="23" t="s">
@@ -5661,7 +5743,7 @@
       <c r="C144" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="D144" s="108">
+      <c r="D144" s="92">
         <v>0.75</v>
       </c>
       <c r="E144" s="24" t="s">
@@ -5673,7 +5755,7 @@
       </c>
     </row>
     <row r="145" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A145" s="105">
+      <c r="A145" s="89">
         <v>46085</v>
       </c>
       <c r="B145" s="23" t="s">
@@ -5682,7 +5764,7 @@
       <c r="C145" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="D145" s="108">
+      <c r="D145" s="92">
         <v>1</v>
       </c>
       <c r="E145" s="24" t="s">
@@ -5694,7 +5776,7 @@
       </c>
     </row>
     <row r="146" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A146" s="105">
+      <c r="A146" s="89">
         <v>46085</v>
       </c>
       <c r="B146" s="23" t="s">
@@ -5703,7 +5785,7 @@
       <c r="C146" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="D146" s="108">
+      <c r="D146" s="92">
         <v>0.75</v>
       </c>
       <c r="E146" s="24" t="s">
@@ -5715,7 +5797,7 @@
       </c>
     </row>
     <row r="147" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A147" s="105">
+      <c r="A147" s="89">
         <v>46086</v>
       </c>
       <c r="B147" s="23" t="s">
@@ -5724,7 +5806,7 @@
       <c r="C147" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="D147" s="108">
+      <c r="D147" s="92">
         <v>1</v>
       </c>
       <c r="E147" s="24" t="s">
@@ -5736,7 +5818,7 @@
       </c>
     </row>
     <row r="148" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A148" s="105">
+      <c r="A148" s="89">
         <v>46086</v>
       </c>
       <c r="B148" s="23" t="s">
@@ -5745,7 +5827,7 @@
       <c r="C148" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="D148" s="108">
+      <c r="D148" s="92">
         <v>0.5</v>
       </c>
       <c r="E148" s="24" t="s">
@@ -5757,7 +5839,7 @@
       </c>
     </row>
     <row r="149" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A149" s="105">
+      <c r="A149" s="89">
         <v>46087</v>
       </c>
       <c r="B149" s="23" t="s">
@@ -5766,7 +5848,7 @@
       <c r="C149" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="D149" s="108">
+      <c r="D149" s="92">
         <v>0.5</v>
       </c>
       <c r="E149" s="24" t="s">
@@ -5778,7 +5860,7 @@
       </c>
     </row>
     <row r="150" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A150" s="105">
+      <c r="A150" s="89">
         <v>46088</v>
       </c>
       <c r="B150" s="23" t="s">
@@ -5787,7 +5869,7 @@
       <c r="C150" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="D150" s="108">
+      <c r="D150" s="92">
         <v>1</v>
       </c>
       <c r="E150" s="24" t="s">
@@ -5801,7 +5883,7 @@
       </c>
     </row>
     <row r="151" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A151" s="105">
+      <c r="A151" s="89">
         <v>46088</v>
       </c>
       <c r="B151" s="23" t="s">
@@ -5810,7 +5892,7 @@
       <c r="C151" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="D151" s="108">
+      <c r="D151" s="92">
         <v>0.75</v>
       </c>
       <c r="E151" s="24" t="s">
@@ -5824,7 +5906,7 @@
       </c>
     </row>
     <row r="152" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A152" s="105">
+      <c r="A152" s="89">
         <v>46089</v>
       </c>
       <c r="B152" s="23" t="s">
@@ -5833,7 +5915,7 @@
       <c r="C152" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="D152" s="108">
+      <c r="D152" s="92">
         <v>0.75</v>
       </c>
       <c r="E152" s="24" t="s">
@@ -5847,7 +5929,7 @@
       </c>
     </row>
     <row r="153" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A153" s="105">
+      <c r="A153" s="89">
         <v>46089</v>
       </c>
       <c r="B153" s="23" t="s">
@@ -5856,7 +5938,7 @@
       <c r="C153" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="D153" s="108">
+      <c r="D153" s="92">
         <v>0.5</v>
       </c>
       <c r="E153" s="24" t="s">
@@ -5870,7 +5952,7 @@
       </c>
     </row>
     <row r="154" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A154" s="105">
+      <c r="A154" s="89">
         <v>46089</v>
       </c>
       <c r="B154" s="23" t="s">
@@ -5879,7 +5961,7 @@
       <c r="C154" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="D154" s="108">
+      <c r="D154" s="92">
         <v>0.5</v>
       </c>
       <c r="E154" s="24" t="s">
@@ -5893,7 +5975,7 @@
       </c>
     </row>
     <row r="155" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A155" s="105">
+      <c r="A155" s="89">
         <v>46089</v>
       </c>
       <c r="B155" s="23" t="s">
@@ -5902,7 +5984,7 @@
       <c r="C155" s="1" t="s">
         <v>427</v>
       </c>
-      <c r="D155" s="108">
+      <c r="D155" s="92">
         <v>1.5</v>
       </c>
       <c r="E155" s="24" t="s">
@@ -5916,7 +5998,7 @@
       </c>
     </row>
     <row r="156" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A156" s="105">
+      <c r="A156" s="89">
         <v>46090</v>
       </c>
       <c r="B156" s="23" t="s">
@@ -5925,7 +6007,7 @@
       <c r="C156" s="1" t="s">
         <v>427</v>
       </c>
-      <c r="D156" s="108">
+      <c r="D156" s="92">
         <v>1.5</v>
       </c>
       <c r="E156" s="24" t="s">
@@ -5939,7 +6021,7 @@
       </c>
     </row>
     <row r="157" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A157" s="105">
+      <c r="A157" s="89">
         <v>46090</v>
       </c>
       <c r="B157" s="23" t="s">
@@ -5948,7 +6030,7 @@
       <c r="C157" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="D157" s="108">
+      <c r="D157" s="92">
         <v>1</v>
       </c>
       <c r="E157" s="24" t="s">
@@ -5962,7 +6044,7 @@
       </c>
     </row>
     <row r="158" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A158" s="106">
+      <c r="A158" s="90">
         <v>46090</v>
       </c>
       <c r="B158" s="1" t="s">
@@ -5985,7 +6067,7 @@
       </c>
     </row>
     <row r="159" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A159" s="106">
+      <c r="A159" s="90">
         <v>46090</v>
       </c>
       <c r="B159" s="1" t="s">
@@ -6008,7 +6090,7 @@
       </c>
     </row>
     <row r="160" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A160" s="106">
+      <c r="A160" s="90">
         <v>46090</v>
       </c>
       <c r="B160" s="1" t="s">
@@ -6031,7 +6113,7 @@
       </c>
     </row>
     <row r="161" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A161" s="106">
+      <c r="A161" s="90">
         <v>46090</v>
       </c>
       <c r="B161" s="1" t="s">
@@ -6054,7 +6136,7 @@
       </c>
     </row>
     <row r="162" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A162" s="106">
+      <c r="A162" s="90">
         <v>46090</v>
       </c>
       <c r="B162" s="1" t="s">
@@ -6077,16 +6159,16 @@
       </c>
     </row>
     <row r="163" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A163" s="107">
+      <c r="A163" s="91">
         <v>46090</v>
       </c>
-      <c r="B163" s="104" t="s">
+      <c r="B163" s="88" t="s">
         <v>383</v>
       </c>
-      <c r="C163" s="104" t="s">
+      <c r="C163" s="88" t="s">
         <v>43</v>
       </c>
-      <c r="D163" s="110">
+      <c r="D163" s="94">
         <v>0.25</v>
       </c>
       <c r="E163" s="24" t="s">
@@ -6100,16 +6182,16 @@
       </c>
     </row>
     <row r="164" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A164" s="107">
+      <c r="A164" s="91">
         <v>46090</v>
       </c>
-      <c r="B164" s="104" t="s">
+      <c r="B164" s="88" t="s">
         <v>383</v>
       </c>
-      <c r="C164" s="104" t="s">
+      <c r="C164" s="88" t="s">
         <v>128</v>
       </c>
-      <c r="D164" s="110">
+      <c r="D164" s="94">
         <v>0.75</v>
       </c>
       <c r="E164" s="24" t="s">
@@ -6121,27 +6203,485 @@
       </c>
     </row>
     <row r="165" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A165" s="88" t="s">
+      <c r="A165" s="91">
+        <v>46092</v>
+      </c>
+      <c r="B165" s="88" t="s">
+        <v>383</v>
+      </c>
+      <c r="C165" s="88" t="s">
+        <v>20</v>
+      </c>
+      <c r="D165" s="94">
+        <v>1</v>
+      </c>
+      <c r="E165" s="24" t="s">
+        <v>215</v>
+      </c>
+      <c r="F165" s="17" t="s">
+        <v>462</v>
+      </c>
+      <c r="G165" s="20" t="s">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="166" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A166" s="91">
+        <v>46092</v>
+      </c>
+      <c r="B166" s="88" t="s">
+        <v>383</v>
+      </c>
+      <c r="C166" s="88" t="s">
+        <v>128</v>
+      </c>
+      <c r="D166" s="94">
+        <v>0.75</v>
+      </c>
+      <c r="E166" s="24" t="s">
+        <v>215</v>
+      </c>
+      <c r="F166" s="17" t="s">
+        <v>462</v>
+      </c>
+      <c r="G166" s="20" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="167" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A167" s="91">
+        <v>46092</v>
+      </c>
+      <c r="B167" s="88" t="s">
+        <v>383</v>
+      </c>
+      <c r="C167" s="88" t="s">
+        <v>442</v>
+      </c>
+      <c r="D167" s="94">
+        <v>1.25</v>
+      </c>
+      <c r="E167" s="24" t="s">
+        <v>215</v>
+      </c>
+      <c r="F167" s="17" t="s">
+        <v>462</v>
+      </c>
+      <c r="G167" s="20" t="s">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="168" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A168" s="91">
+        <v>46092</v>
+      </c>
+      <c r="B168" s="88" t="s">
+        <v>383</v>
+      </c>
+      <c r="C168" s="88" t="s">
+        <v>20</v>
+      </c>
+      <c r="D168" s="94">
+        <v>1</v>
+      </c>
+      <c r="E168" s="24" t="s">
+        <v>215</v>
+      </c>
+      <c r="F168" s="17" t="s">
+        <v>462</v>
+      </c>
+      <c r="G168" s="20" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="169" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A169" s="91">
+        <v>46094</v>
+      </c>
+      <c r="B169" s="88" t="s">
+        <v>383</v>
+      </c>
+      <c r="C169" s="88" t="s">
+        <v>128</v>
+      </c>
+      <c r="D169" s="94">
+        <v>0.75</v>
+      </c>
+      <c r="E169" s="24" t="s">
+        <v>215</v>
+      </c>
+      <c r="F169" s="17" t="s">
+        <v>462</v>
+      </c>
+      <c r="G169" s="20" t="s">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="170" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A170" s="91">
+        <v>46094</v>
+      </c>
+      <c r="B170" s="88" t="s">
+        <v>383</v>
+      </c>
+      <c r="C170" s="88" t="s">
+        <v>20</v>
+      </c>
+      <c r="D170" s="94">
+        <v>1</v>
+      </c>
+      <c r="E170" s="24" t="s">
+        <v>215</v>
+      </c>
+      <c r="F170" s="17" t="s">
+        <v>462</v>
+      </c>
+      <c r="G170" s="20" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="171" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A171" s="91">
+        <v>46094</v>
+      </c>
+      <c r="B171" s="88" t="s">
+        <v>383</v>
+      </c>
+      <c r="C171" s="88" t="s">
+        <v>442</v>
+      </c>
+      <c r="D171" s="94">
+        <v>1.25</v>
+      </c>
+      <c r="E171" s="24" t="s">
+        <v>215</v>
+      </c>
+      <c r="F171" s="17" t="s">
+        <v>462</v>
+      </c>
+      <c r="G171" s="20" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="172" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A172" s="91">
+        <v>46094</v>
+      </c>
+      <c r="B172" s="88" t="s">
+        <v>383</v>
+      </c>
+      <c r="C172" s="88" t="s">
+        <v>128</v>
+      </c>
+      <c r="D172" s="94">
+        <v>0.75</v>
+      </c>
+      <c r="E172" s="24" t="s">
+        <v>215</v>
+      </c>
+      <c r="F172" s="17" t="s">
+        <v>462</v>
+      </c>
+      <c r="G172" s="20" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="173" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A173" s="91">
+        <v>46096</v>
+      </c>
+      <c r="B173" s="88" t="s">
+        <v>383</v>
+      </c>
+      <c r="C173" s="88" t="s">
+        <v>128</v>
+      </c>
+      <c r="D173" s="94">
+        <v>0.75</v>
+      </c>
+      <c r="E173" s="24" t="s">
+        <v>215</v>
+      </c>
+      <c r="F173" s="17" t="s">
+        <v>462</v>
+      </c>
+      <c r="G173" s="20" t="s">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="174" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A174" s="91">
+        <v>46096</v>
+      </c>
+      <c r="B174" s="88" t="s">
+        <v>383</v>
+      </c>
+      <c r="C174" s="88" t="s">
+        <v>74</v>
+      </c>
+      <c r="D174" s="94">
+        <v>0.5</v>
+      </c>
+      <c r="E174" s="24" t="s">
+        <v>215</v>
+      </c>
+      <c r="F174" s="17" t="s">
+        <v>462</v>
+      </c>
+      <c r="G174" s="20" t="s">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="175" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A175" s="91">
+        <v>46096</v>
+      </c>
+      <c r="B175" s="88" t="s">
+        <v>383</v>
+      </c>
+      <c r="C175" s="88" t="s">
+        <v>128</v>
+      </c>
+      <c r="D175" s="94">
+        <v>0.75</v>
+      </c>
+      <c r="E175" s="24" t="s">
+        <v>215</v>
+      </c>
+      <c r="F175" s="17" t="s">
+        <v>462</v>
+      </c>
+      <c r="G175" s="20" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="176" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A176" s="91">
+        <v>46096</v>
+      </c>
+      <c r="B176" s="88" t="s">
+        <v>383</v>
+      </c>
+      <c r="C176" s="88" t="s">
+        <v>74</v>
+      </c>
+      <c r="D176" s="94">
+        <v>0.5</v>
+      </c>
+      <c r="E176" s="24" t="s">
+        <v>215</v>
+      </c>
+      <c r="F176" s="17" t="s">
+        <v>462</v>
+      </c>
+      <c r="G176" s="20" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="177" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A177" s="91">
+        <v>46097</v>
+      </c>
+      <c r="B177" s="88" t="s">
+        <v>453</v>
+      </c>
+      <c r="C177" s="88" t="s">
+        <v>20</v>
+      </c>
+      <c r="D177" s="94">
+        <v>1</v>
+      </c>
+      <c r="E177" s="24" t="s">
+        <v>216</v>
+      </c>
+      <c r="F177" s="17" t="s">
+        <v>463</v>
+      </c>
+      <c r="G177" s="20" t="s">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="178" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A178" s="91">
+        <v>46097</v>
+      </c>
+      <c r="B178" s="88" t="s">
+        <v>453</v>
+      </c>
+      <c r="C178" s="88" t="s">
+        <v>442</v>
+      </c>
+      <c r="D178" s="94">
+        <v>1.25</v>
+      </c>
+      <c r="E178" s="24" t="s">
+        <v>216</v>
+      </c>
+      <c r="F178" s="17" t="s">
+        <v>463</v>
+      </c>
+      <c r="G178" s="20" t="s">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="179" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A179" s="91">
+        <v>46097</v>
+      </c>
+      <c r="B179" s="88" t="s">
+        <v>453</v>
+      </c>
+      <c r="C179" s="88" t="s">
+        <v>74</v>
+      </c>
+      <c r="D179" s="94">
+        <v>0.5</v>
+      </c>
+      <c r="E179" s="24" t="s">
+        <v>216</v>
+      </c>
+      <c r="F179" s="17" t="s">
+        <v>463</v>
+      </c>
+      <c r="G179" s="20" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="180" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A180" s="91">
+        <v>46097</v>
+      </c>
+      <c r="B180" s="88" t="s">
+        <v>453</v>
+      </c>
+      <c r="C180" s="88" t="s">
+        <v>427</v>
+      </c>
+      <c r="D180" s="94">
+        <v>1.5</v>
+      </c>
+      <c r="E180" s="24" t="s">
+        <v>217</v>
+      </c>
+      <c r="F180" s="17" t="s">
+        <v>464</v>
+      </c>
+      <c r="G180" s="20" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="181" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A181" s="91">
+        <v>46097</v>
+      </c>
+      <c r="B181" s="88" t="s">
+        <v>453</v>
+      </c>
+      <c r="C181" s="88" t="s">
+        <v>458</v>
+      </c>
+      <c r="D181" s="94">
+        <v>1.75</v>
+      </c>
+      <c r="E181" s="24" t="s">
+        <v>217</v>
+      </c>
+      <c r="F181" s="17" t="s">
+        <v>464</v>
+      </c>
+      <c r="G181" s="20" t="s">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="182" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A182" s="91">
+        <v>46097</v>
+      </c>
+      <c r="B182" s="88" t="s">
+        <v>453</v>
+      </c>
+      <c r="C182" s="88" t="s">
+        <v>427</v>
+      </c>
+      <c r="D182" s="94">
+        <v>1.5</v>
+      </c>
+      <c r="E182" s="24" t="s">
+        <v>217</v>
+      </c>
+      <c r="F182" s="17" t="s">
+        <v>464</v>
+      </c>
+      <c r="G182" s="20" t="s">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="183" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A183" s="91">
+        <v>46097</v>
+      </c>
+      <c r="B183" s="88" t="s">
+        <v>453</v>
+      </c>
+      <c r="C183" s="88" t="s">
+        <v>74</v>
+      </c>
+      <c r="D183" s="94">
+        <v>0.5</v>
+      </c>
+      <c r="E183" s="24" t="s">
+        <v>217</v>
+      </c>
+      <c r="F183" s="17" t="s">
+        <v>464</v>
+      </c>
+      <c r="G183" s="20" t="s">
+        <v>461</v>
+      </c>
+    </row>
+    <row r="184" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A184" s="91">
+        <v>46097</v>
+      </c>
+      <c r="B184" s="88" t="s">
+        <v>383</v>
+      </c>
+      <c r="C184" s="88" t="s">
+        <v>128</v>
+      </c>
+      <c r="D184" s="94">
+        <v>0.75</v>
+      </c>
+      <c r="E184" s="24" t="s">
+        <v>37</v>
+      </c>
+      <c r="F184" s="17"/>
+      <c r="G184" s="20" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="185" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A185" s="95" t="s">
         <v>137</v>
       </c>
-      <c r="B165" s="89"/>
-      <c r="C165" s="89"/>
-      <c r="D165" s="90"/>
-      <c r="E165" s="73">
-        <f>SUM(D6:D164)</f>
-        <v>119.85</v>
-      </c>
-      <c r="F165" s="18"/>
-      <c r="G165" s="21"/>
+      <c r="B185" s="96"/>
+      <c r="C185" s="96"/>
+      <c r="D185" s="97"/>
+      <c r="E185" s="73">
+        <f>SUM(D6:D184)</f>
+        <v>138.85</v>
+      </c>
+      <c r="F185" s="18"/>
+      <c r="G185" s="21"/>
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A165:D165"/>
+    <mergeCell ref="A185:D185"/>
     <mergeCell ref="A3:G3"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A1:G1"/>
   </mergeCells>
-  <conditionalFormatting sqref="E6:E217">
+  <conditionalFormatting sqref="E6:E237">
     <cfRule type="cellIs" dxfId="20" priority="1" operator="equal">
       <formula>"0: Environment Setup"</formula>
     </cfRule>
@@ -6214,7 +6754,7 @@
           <x14:formula1>
             <xm:f>Categories!$A$4:$A$25</xm:f>
           </x14:formula1>
-          <xm:sqref>E6:E217</xm:sqref>
+          <xm:sqref>E6:E237</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -6232,31 +6772,31 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="22.8" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="103" t="s">
+      <c r="A1" s="110" t="s">
         <v>138</v>
       </c>
-      <c r="B1" s="96"/>
-      <c r="C1" s="96"/>
-      <c r="D1" s="96"/>
-      <c r="E1" s="96"/>
-      <c r="F1" s="96"/>
-      <c r="G1" s="96"/>
-      <c r="H1" s="96"/>
-      <c r="I1" s="96"/>
-      <c r="J1" s="96"/>
-      <c r="K1" s="96"/>
-      <c r="L1" s="96"/>
-      <c r="M1" s="96"/>
-      <c r="N1" s="96"/>
+      <c r="B1" s="103"/>
+      <c r="C1" s="103"/>
+      <c r="D1" s="103"/>
+      <c r="E1" s="103"/>
+      <c r="F1" s="103"/>
+      <c r="G1" s="103"/>
+      <c r="H1" s="103"/>
+      <c r="I1" s="103"/>
+      <c r="J1" s="103"/>
+      <c r="K1" s="103"/>
+      <c r="L1" s="103"/>
+      <c r="M1" s="103"/>
+      <c r="N1" s="103"/>
     </row>
     <row r="3" spans="1:14" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="100" t="s">
+      <c r="A3" s="107" t="s">
         <v>139</v>
       </c>
-      <c r="B3" s="96"/>
-      <c r="C3" s="96"/>
-      <c r="D3" s="96"/>
-      <c r="E3" s="96"/>
+      <c r="B3" s="103"/>
+      <c r="C3" s="103"/>
+      <c r="D3" s="103"/>
+      <c r="E3" s="103"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4" s="33" t="s">
@@ -6344,7 +6884,7 @@
       </c>
       <c r="D8" s="37">
         <f>SUM(B56:B60)</f>
-        <v>26.5</v>
+        <v>36.75</v>
       </c>
       <c r="E8" s="38">
         <f t="shared" si="0"/>
@@ -6363,11 +6903,11 @@
       </c>
       <c r="D9" s="37">
         <f>SUM(B61:B62)</f>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="E9" s="38">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.3">
@@ -6401,11 +6941,11 @@
       </c>
       <c r="D11" s="37">
         <f>SUM(B65)</f>
-        <v>14</v>
+        <v>14.75</v>
       </c>
       <c r="E11" s="38">
         <f t="shared" si="0"/>
-        <v>0.77777777777777779</v>
+        <v>0.81944444444444442</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.3">
@@ -6419,30 +6959,30 @@
       </c>
       <c r="D12" s="54">
         <f>SUM(D5:D11)</f>
-        <v>96.6</v>
+        <v>115.6</v>
       </c>
       <c r="E12" s="55">
         <f>IF(C12=0,0,D12/C12)</f>
-        <v>0.81864406779661014</v>
+        <v>0.97966101694915253</v>
       </c>
     </row>
     <row r="14" spans="1:14" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="101" t="s">
+      <c r="A14" s="108" t="s">
         <v>152</v>
       </c>
-      <c r="B14" s="102"/>
-      <c r="C14" s="102"/>
-      <c r="D14" s="102"/>
-      <c r="E14" s="102"/>
-      <c r="F14" s="102"/>
-      <c r="G14" s="102"/>
-      <c r="H14" s="102"/>
-      <c r="I14" s="102"/>
-      <c r="J14" s="102"/>
-      <c r="K14" s="102"/>
-      <c r="L14" s="102"/>
-      <c r="M14" s="102"/>
-      <c r="N14" s="102"/>
+      <c r="B14" s="109"/>
+      <c r="C14" s="109"/>
+      <c r="D14" s="109"/>
+      <c r="E14" s="109"/>
+      <c r="F14" s="109"/>
+      <c r="G14" s="109"/>
+      <c r="H14" s="109"/>
+      <c r="I14" s="109"/>
+      <c r="J14" s="109"/>
+      <c r="K14" s="109"/>
+      <c r="L14" s="109"/>
+      <c r="M14" s="109"/>
+      <c r="N14" s="109"/>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A15" s="33" t="s">
@@ -7148,7 +7688,7 @@
       </c>
       <c r="B59" s="37">
         <f>SUMIF('Work Log'!E:E,"3D: Health Education Library",'Work Log'!D:D)</f>
-        <v>0</v>
+        <v>10.25</v>
       </c>
       <c r="C59" s="3"/>
     </row>
@@ -7168,7 +7708,7 @@
       </c>
       <c r="B61" s="37">
         <f>SUMIF('Work Log'!E:E,"4A: System Analytics Data",'Work Log'!D:D)</f>
-        <v>0</v>
+        <v>2.75</v>
       </c>
       <c r="C61" s="3"/>
     </row>
@@ -7178,7 +7718,7 @@
       </c>
       <c r="B62" s="37">
         <f>SUMIF('Work Log'!E:E,"4B: System Analytics Dashboard",'Work Log'!D:D)</f>
-        <v>0</v>
+        <v>5.25</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.3">
@@ -7205,7 +7745,7 @@
       </c>
       <c r="B65" s="37">
         <f>SUMIF('Work Log'!E:E,"6: Documentation + Submission",'Work Log'!D:D)</f>
-        <v>14</v>
+        <v>14.75</v>
       </c>
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.3">
@@ -7230,9 +7770,9 @@
       <c r="A68" s="51" t="s">
         <v>151</v>
       </c>
-      <c r="B68" s="109">
+      <c r="B68" s="93">
         <f>SUM(B46:B67)</f>
-        <v>119.85000000000001</v>
+        <v>138.85000000000002</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated Work Log and uploaded Progress Report 5
</commit_message>
<xml_diff>
--- a/DocumentsAndReports/worklog/WorkLog_DesmondChua_W26_4495_S2.xlsx
+++ b/DocumentsAndReports/worklog/WorkLog_DesmondChua_W26_4495_S2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d4f25ae689476683/Desmond_New/BC-Health-Platform/DocumentsAndReports/worklog/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="182" documentId="8_{08655895-4010-492B-B73A-F5D36A9F8AF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DBECE850-859A-40A1-B437-F926111F1D88}"/>
+  <xr:revisionPtr revIDLastSave="189" documentId="8_{08655895-4010-492B-B73A-F5D36A9F8AF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8130E292-2780-4531-992B-4C84406774B9}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1129" uniqueCount="466">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1244" uniqueCount="502">
   <si>
     <t>CSIS 4495 - Applied Research Project</t>
   </si>
@@ -1433,6 +1433,114 @@
   </si>
   <si>
     <t>Prepared Progress Report 4; updated commit history, work log entries, and timeline for PR4 reporting period (Mar 10–16); added screenshots and submitted to Blackboard</t>
+  </si>
+  <si>
+    <t>Sprint 5</t>
+  </si>
+  <si>
+    <t>5A: Automated Testing Suite</t>
+  </si>
+  <si>
+    <t>5A.1</t>
+  </si>
+  <si>
+    <t>Sprint 5A scope planning: Decided to drop Community Pulse (web scraping) feature and focus on automated testing suite. Drafted scope decision rationale and sent email to Prof. Priya explaining the scope change and requesting absence from class for job interview</t>
+  </si>
+  <si>
+    <t>Sprint 5A.1: Designed tests/ folder architecture — unit/, integration/, ui/, property/ sub-packages. Created all init.py files, conftest.py with test_db (in-memory SQLite fixture with yield teardown) and test_user fixtures, TEST_REGISTER.md with table header</t>
+  </si>
+  <si>
+    <t>Sprint 5A.1 cleanup: Identified and removed old ad-hoc test scripts (test_openai.py, test_predict.py, test_rules.py) from Implementation/tests/ — superseded by new proper pytest suite at root tests/ folder</t>
+  </si>
+  <si>
+    <t>5A.2</t>
+  </si>
+  <si>
+    <t>Sprint 5A.2: Read auth.py source code to understand exact function signatures (hash_password, verify_password, validate_password_strength, validate_email, require_authentication). Designed 10 test cases across 4 logical groups: Registration, Login, Security, Session</t>
+  </si>
+  <si>
+    <t>Sprint 5A.2: Wrote test_auth.py — 10 unit tests for authentication module. Used conftest.py test_db fixture for all database operations, unittest.mock for Streamlit session_state and st.switch_page. Verified all 10 tests pass: 10/10 passed in 4.38s</t>
+  </si>
+  <si>
+    <t>5A.3</t>
+  </si>
+  <si>
+    <t>Sprint 5A.3 analysis: Read rules.py to confirm check_critical_symptoms() signature, return dict structure, 14-rule count, match types (any vs all), case-insensitive matching behaviour before writing tests</t>
+  </si>
+  <si>
+    <t>Sprint 5A.3: Wrote test_ctas_rules.py — 23 unit tests across 3 groups: 14 parametrized positive detection tests (one per CTAS rule), 5 negative pass-through tests, 4 edge case tests (mixed case, None input, large lists, single keyword). All 23 passing</t>
+  </si>
+  <si>
+    <t>5A.4</t>
+  </si>
+  <si>
+    <t>Sprint 5A.4 analysis: Read database.py (690 lines) — confirmed all CRUD function signatures, return types, table schema, and connection pattern (get_connection() called internally — requires unittest.mock.patch to redirect to test DB)</t>
+  </si>
+  <si>
+    <t>Sprint 5A.4: Wrote test_database.py — 12 unit tests across 3 groups: 5 User CRUD tests, 5 Assessment CRUD tests, 2 Data Integrity tests. Patched get_connection() with test DB factory. Verified user isolation (TC-DB-11) and correct FK constraint handling. All 12 passing</t>
+  </si>
+  <si>
+    <t>5A.5</t>
+  </si>
+  <si>
+    <t>Sprint 5A.5 analysis: Confirmed ML layer lives in chatbot.py (not ml_model.py). Read model.pkl and model_metadata.json directly — identified feature vector building logic, 70% confidence threshold location, predict_proba() call pattern</t>
+  </si>
+  <si>
+    <t>Sprint 5A.5: Wrote test_ml_model.py — 12 unit tests across 4 groups: model loading (2), confidence threshold (3), input handling (4), output validation (3). Loaded real model.pkl directly without Streamlit. UTI symptoms achieved 100% confidence. All 12 passing</t>
+  </si>
+  <si>
+    <t>5A.6</t>
+  </si>
+  <si>
+    <t>Sprint 5A.6 analysis: Read chatbot.py — confirmed run_assessment() layer sequence (OpenAI → CTAS → ML), all 4 return statuses and their dict keys, patch target (components.chatbot.extract_symptoms — patch where used not where defined)</t>
+  </si>
+  <si>
+    <t>Sprint 5A.6: Wrote test_pipeline.py — 6 integration tests. Mocked both extract_symptoms() and get_openai_fallback_guidance(). Tested emergency circuit breaker, ML prediction path, OpenAI fallback path, safety invariants. All 6 passing in 3.74s</t>
+  </si>
+  <si>
+    <t>5A.7</t>
+  </si>
+  <si>
+    <t>Sprint 5A.7 analysis: Confirmed extract_symptoms() return dict key is 'symptoms' (not 'extracted_symptoms'). Confirmed all mock return structures for 6 clinical scenarios before writing tests</t>
+  </si>
+  <si>
+    <t>Sprint 5A.7: Wrote test_chatbot_scenarios.py — 6 integration tests covering cardiac emergency, stroke emergency, UTI ML prediction, vague symptom fallback, emergency override safety, minimal input edge case. All 6 passing on first run</t>
+  </si>
+  <si>
+    <t>5A.8</t>
+  </si>
+  <si>
+    <t>Sprint 5A.8 analysis: Read 3_My_Dashboard.py — confirmed session_state keys, data source (get_user_assessments via components.database), 4 stat cards as custom HTML st.markdown (not st.metric), 2 selectboxes, CWD dependency for assets/logo.png</t>
+  </si>
+  <si>
+    <t>Sprint 5A.8: Wrote test_dashboard_apptest.py — 8 headless UI tests using Streamlit AppTest. Implemented _run_dashboard() helper with os.chdir(SRC_DIR) pattern. Verified stat card headers, selectbox options (All Time, Last 3 Months, All Urgency Levels), user data isolation. All 8 passing</t>
+  </si>
+  <si>
+    <t>5A.9</t>
+  </si>
+  <si>
+    <t>Sprint 5A.9 analysis: Read 2_Symptom_Assessment.py — confirmed session_state keys, process_multiturn_message() as primary function to mock (not run_assessment()), AppTest chat input syntax (at.chat_input[0].set_value().run()), _submit_chat() helper pattern needed</t>
+  </si>
+  <si>
+    <t>Sprint 5A.9: Wrote test_chatbot_apptest.py — 8 headless UI tests. Implemented _run_chatbot() and _submit_chat() helpers with patch re-application on rerun. Tested warning banner, welcome message personalisation, ML response, emergency response, auth guard. All 8 passing</t>
+  </si>
+  <si>
+    <t>5A.10</t>
+  </si>
+  <si>
+    <t>Sprint 5A.10 analysis: Confirmed Hypothesis installed (6.151.9). Read auth.py and rules.py to verify exact validation rules — password requires letter + digit (not uppercase + lowercase separately). Corrected strategy before writing</t>
+  </si>
+  <si>
+    <t>Sprint 5A.10: Wrote test_fuzz_hypothesis.py — 10 property-based tests using Hypothesis. 1,000 total fuzz inputs (100 per test). Covered password fuzzing (3 tests), email fuzzing (3 tests), CTAS rules fuzzing (3 tests), database fuzzing (1 test). All 10 passing</t>
+  </si>
+  <si>
+    <t>5A.11</t>
+  </si>
+  <si>
+    <t>Sprint 5A.11: Ran full test suite from project root — 79 tests across unit, integration, property folders all passing in 20.89s. UI tests confirmed passing individually (16 tests). Took screenshots for progress report documentation</t>
+  </si>
+  <si>
+    <t>Git commits: All Sprint 5A tasks committed with granular messages (5A.1 through 5A.11) and pushed to GitHub main branch</t>
   </si>
 </sst>
 </file>
@@ -1574,7 +1682,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="26">
+  <fills count="27">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1703,6 +1811,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFB7E4CF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="8">
     <border>
@@ -1809,7 +1923,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="111">
+  <cellXfs count="112">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2048,6 +2162,9 @@
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="26" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2524,7 +2641,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G185"/>
+  <dimension ref="A1:G208"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -6644,7 +6761,7 @@
         <v>46097</v>
       </c>
       <c r="B184" s="88" t="s">
-        <v>383</v>
+        <v>453</v>
       </c>
       <c r="C184" s="88" t="s">
         <v>128</v>
@@ -6661,27 +6778,556 @@
       </c>
     </row>
     <row r="185" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A185" s="95" t="s">
+      <c r="A185" s="91">
+        <v>46098</v>
+      </c>
+      <c r="B185" s="88" t="s">
+        <v>466</v>
+      </c>
+      <c r="C185" s="88" t="s">
+        <v>20</v>
+      </c>
+      <c r="D185" s="94">
+        <v>1</v>
+      </c>
+      <c r="E185" s="111" t="s">
+        <v>467</v>
+      </c>
+      <c r="F185" s="17" t="s">
+        <v>468</v>
+      </c>
+      <c r="G185" s="20" t="s">
+        <v>469</v>
+      </c>
+    </row>
+    <row r="186" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A186" s="91">
+        <v>46098</v>
+      </c>
+      <c r="B186" s="88" t="s">
+        <v>466</v>
+      </c>
+      <c r="C186" s="88" t="s">
+        <v>128</v>
+      </c>
+      <c r="D186" s="94">
+        <v>0.75</v>
+      </c>
+      <c r="E186" s="111" t="s">
+        <v>467</v>
+      </c>
+      <c r="F186" s="17" t="s">
+        <v>468</v>
+      </c>
+      <c r="G186" s="20" t="s">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="187" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A187" s="91">
+        <v>46098</v>
+      </c>
+      <c r="B187" s="88" t="s">
+        <v>466</v>
+      </c>
+      <c r="C187" s="88" t="s">
+        <v>74</v>
+      </c>
+      <c r="D187" s="94">
+        <v>0.5</v>
+      </c>
+      <c r="E187" s="111" t="s">
+        <v>467</v>
+      </c>
+      <c r="F187" s="17" t="s">
+        <v>468</v>
+      </c>
+      <c r="G187" s="20" t="s">
+        <v>471</v>
+      </c>
+    </row>
+    <row r="188" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A188" s="91">
+        <v>46100</v>
+      </c>
+      <c r="B188" s="88" t="s">
+        <v>466</v>
+      </c>
+      <c r="C188" s="88" t="s">
+        <v>20</v>
+      </c>
+      <c r="D188" s="94">
+        <v>1</v>
+      </c>
+      <c r="E188" s="111" t="s">
+        <v>467</v>
+      </c>
+      <c r="F188" s="17" t="s">
+        <v>472</v>
+      </c>
+      <c r="G188" s="20" t="s">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="189" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A189" s="91">
+        <v>46100</v>
+      </c>
+      <c r="B189" s="88" t="s">
+        <v>466</v>
+      </c>
+      <c r="C189" s="88" t="s">
+        <v>442</v>
+      </c>
+      <c r="D189" s="94">
+        <v>1.25</v>
+      </c>
+      <c r="E189" s="111" t="s">
+        <v>467</v>
+      </c>
+      <c r="F189" s="17" t="s">
+        <v>472</v>
+      </c>
+      <c r="G189" s="20" t="s">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="190" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A190" s="91">
+        <v>46100</v>
+      </c>
+      <c r="B190" s="88" t="s">
+        <v>466</v>
+      </c>
+      <c r="C190" s="88" t="s">
+        <v>74</v>
+      </c>
+      <c r="D190" s="94">
+        <v>0.5</v>
+      </c>
+      <c r="E190" s="111" t="s">
+        <v>467</v>
+      </c>
+      <c r="F190" s="17" t="s">
+        <v>475</v>
+      </c>
+      <c r="G190" s="20" t="s">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="191" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A191" s="91">
+        <v>46102</v>
+      </c>
+      <c r="B191" s="88" t="s">
+        <v>466</v>
+      </c>
+      <c r="C191" s="88" t="s">
+        <v>427</v>
+      </c>
+      <c r="D191" s="94">
+        <v>1.5</v>
+      </c>
+      <c r="E191" s="111" t="s">
+        <v>467</v>
+      </c>
+      <c r="F191" s="17" t="s">
+        <v>475</v>
+      </c>
+      <c r="G191" s="20" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="192" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A192" s="91">
+        <v>46102</v>
+      </c>
+      <c r="B192" s="88" t="s">
+        <v>466</v>
+      </c>
+      <c r="C192" s="88" t="s">
+        <v>128</v>
+      </c>
+      <c r="D192" s="94">
+        <v>0.75</v>
+      </c>
+      <c r="E192" s="111" t="s">
+        <v>467</v>
+      </c>
+      <c r="F192" s="17" t="s">
+        <v>478</v>
+      </c>
+      <c r="G192" s="20" t="s">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="193" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A193" s="91">
+        <v>46102</v>
+      </c>
+      <c r="B193" s="88" t="s">
+        <v>466</v>
+      </c>
+      <c r="C193" s="88" t="s">
+        <v>442</v>
+      </c>
+      <c r="D193" s="94">
+        <v>1.25</v>
+      </c>
+      <c r="E193" s="111" t="s">
+        <v>467</v>
+      </c>
+      <c r="F193" s="17" t="s">
+        <v>478</v>
+      </c>
+      <c r="G193" s="20" t="s">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="194" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A194" s="91">
+        <v>46102</v>
+      </c>
+      <c r="B194" s="88" t="s">
+        <v>466</v>
+      </c>
+      <c r="C194" s="88" t="s">
+        <v>128</v>
+      </c>
+      <c r="D194" s="94">
+        <v>0.75</v>
+      </c>
+      <c r="E194" s="111" t="s">
+        <v>467</v>
+      </c>
+      <c r="F194" s="17" t="s">
+        <v>481</v>
+      </c>
+      <c r="G194" s="20" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="195" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A195" s="91">
+        <v>46102</v>
+      </c>
+      <c r="B195" s="88" t="s">
+        <v>466</v>
+      </c>
+      <c r="C195" s="88" t="s">
+        <v>442</v>
+      </c>
+      <c r="D195" s="94">
+        <v>1.25</v>
+      </c>
+      <c r="E195" s="111" t="s">
+        <v>467</v>
+      </c>
+      <c r="F195" s="17" t="s">
+        <v>481</v>
+      </c>
+      <c r="G195" s="20" t="s">
+        <v>483</v>
+      </c>
+    </row>
+    <row r="196" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A196" s="91">
+        <v>46103</v>
+      </c>
+      <c r="B196" s="88" t="s">
+        <v>466</v>
+      </c>
+      <c r="C196" s="88" t="s">
+        <v>128</v>
+      </c>
+      <c r="D196" s="94">
+        <v>0.75</v>
+      </c>
+      <c r="E196" s="111" t="s">
+        <v>467</v>
+      </c>
+      <c r="F196" s="17" t="s">
+        <v>484</v>
+      </c>
+      <c r="G196" s="20" t="s">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="197" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A197" s="91">
+        <v>46103</v>
+      </c>
+      <c r="B197" s="88" t="s">
+        <v>466</v>
+      </c>
+      <c r="C197" s="88" t="s">
+        <v>442</v>
+      </c>
+      <c r="D197" s="94">
+        <v>1.25</v>
+      </c>
+      <c r="E197" s="111" t="s">
+        <v>467</v>
+      </c>
+      <c r="F197" s="17" t="s">
+        <v>484</v>
+      </c>
+      <c r="G197" s="20" t="s">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="198" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A198" s="91">
+        <v>46104</v>
+      </c>
+      <c r="B198" s="88" t="s">
+        <v>466</v>
+      </c>
+      <c r="C198" s="88" t="s">
+        <v>128</v>
+      </c>
+      <c r="D198" s="94">
+        <v>0.75</v>
+      </c>
+      <c r="E198" s="111" t="s">
+        <v>467</v>
+      </c>
+      <c r="F198" s="17" t="s">
+        <v>487</v>
+      </c>
+      <c r="G198" s="20" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="199" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A199" s="91">
+        <v>46104</v>
+      </c>
+      <c r="B199" s="88" t="s">
+        <v>466</v>
+      </c>
+      <c r="C199" s="88" t="s">
+        <v>442</v>
+      </c>
+      <c r="D199" s="94">
+        <v>1.25</v>
+      </c>
+      <c r="E199" s="111" t="s">
+        <v>467</v>
+      </c>
+      <c r="F199" s="17" t="s">
+        <v>487</v>
+      </c>
+      <c r="G199" s="20" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="200" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A200" s="91">
+        <v>46104</v>
+      </c>
+      <c r="B200" s="88" t="s">
+        <v>466</v>
+      </c>
+      <c r="C200" s="88" t="s">
+        <v>128</v>
+      </c>
+      <c r="D200" s="94">
+        <v>0.75</v>
+      </c>
+      <c r="E200" s="111" t="s">
+        <v>467</v>
+      </c>
+      <c r="F200" s="17" t="s">
+        <v>490</v>
+      </c>
+      <c r="G200" s="20" t="s">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="201" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A201" s="91">
+        <v>46104</v>
+      </c>
+      <c r="B201" s="88" t="s">
+        <v>466</v>
+      </c>
+      <c r="C201" s="88" t="s">
+        <v>427</v>
+      </c>
+      <c r="D201" s="94">
+        <v>1.5</v>
+      </c>
+      <c r="E201" s="111" t="s">
+        <v>467</v>
+      </c>
+      <c r="F201" s="17" t="s">
+        <v>490</v>
+      </c>
+      <c r="G201" s="20" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="202" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A202" s="91">
+        <v>46104</v>
+      </c>
+      <c r="B202" s="88" t="s">
+        <v>466</v>
+      </c>
+      <c r="C202" s="88" t="s">
+        <v>128</v>
+      </c>
+      <c r="D202" s="94">
+        <v>0.75</v>
+      </c>
+      <c r="E202" s="111" t="s">
+        <v>467</v>
+      </c>
+      <c r="F202" s="17" t="s">
+        <v>493</v>
+      </c>
+      <c r="G202" s="20" t="s">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="203" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A203" s="91">
+        <v>46104</v>
+      </c>
+      <c r="B203" s="88" t="s">
+        <v>466</v>
+      </c>
+      <c r="C203" s="88" t="s">
+        <v>427</v>
+      </c>
+      <c r="D203" s="94">
+        <v>1.5</v>
+      </c>
+      <c r="E203" s="111" t="s">
+        <v>467</v>
+      </c>
+      <c r="F203" s="17" t="s">
+        <v>493</v>
+      </c>
+      <c r="G203" s="20" t="s">
+        <v>495</v>
+      </c>
+    </row>
+    <row r="204" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A204" s="91">
+        <v>46104</v>
+      </c>
+      <c r="B204" s="88" t="s">
+        <v>466</v>
+      </c>
+      <c r="C204" s="88" t="s">
+        <v>128</v>
+      </c>
+      <c r="D204" s="94">
+        <v>0.75</v>
+      </c>
+      <c r="E204" s="111" t="s">
+        <v>467</v>
+      </c>
+      <c r="F204" s="17" t="s">
+        <v>496</v>
+      </c>
+      <c r="G204" s="20" t="s">
+        <v>497</v>
+      </c>
+    </row>
+    <row r="205" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A205" s="91">
+        <v>46104</v>
+      </c>
+      <c r="B205" s="88" t="s">
+        <v>466</v>
+      </c>
+      <c r="C205" s="88" t="s">
+        <v>442</v>
+      </c>
+      <c r="D205" s="94">
+        <v>1.25</v>
+      </c>
+      <c r="E205" s="111" t="s">
+        <v>467</v>
+      </c>
+      <c r="F205" s="17" t="s">
+        <v>496</v>
+      </c>
+      <c r="G205" s="20" t="s">
+        <v>498</v>
+      </c>
+    </row>
+    <row r="206" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A206" s="91">
+        <v>46104</v>
+      </c>
+      <c r="B206" s="88" t="s">
+        <v>466</v>
+      </c>
+      <c r="C206" s="88" t="s">
+        <v>74</v>
+      </c>
+      <c r="D206" s="94">
+        <v>0.5</v>
+      </c>
+      <c r="E206" s="111" t="s">
+        <v>467</v>
+      </c>
+      <c r="F206" s="17" t="s">
+        <v>499</v>
+      </c>
+      <c r="G206" s="20" t="s">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="207" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A207" s="91">
+        <v>46104</v>
+      </c>
+      <c r="B207" s="88" t="s">
+        <v>466</v>
+      </c>
+      <c r="C207" s="88" t="s">
+        <v>43</v>
+      </c>
+      <c r="D207" s="94">
+        <v>0.25</v>
+      </c>
+      <c r="E207" s="24" t="s">
+        <v>37</v>
+      </c>
+      <c r="F207" s="17" t="s">
+        <v>499</v>
+      </c>
+      <c r="G207" s="20" t="s">
+        <v>501</v>
+      </c>
+    </row>
+    <row r="208" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A208" s="95" t="s">
         <v>137</v>
       </c>
-      <c r="B185" s="96"/>
-      <c r="C185" s="96"/>
-      <c r="D185" s="97"/>
-      <c r="E185" s="73">
-        <f>SUM(D6:D184)</f>
-        <v>138.85</v>
-      </c>
-      <c r="F185" s="18"/>
-      <c r="G185" s="21"/>
+      <c r="B208" s="96"/>
+      <c r="C208" s="96"/>
+      <c r="D208" s="97"/>
+      <c r="E208" s="73">
+        <f>SUM(D6:D207)</f>
+        <v>160.6</v>
+      </c>
+      <c r="F208" s="18"/>
+      <c r="G208" s="21"/>
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A185:D185"/>
+    <mergeCell ref="A208:D208"/>
     <mergeCell ref="A3:G3"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A1:G1"/>
   </mergeCells>
-  <conditionalFormatting sqref="E6:E237">
+  <conditionalFormatting sqref="E6:E260">
     <cfRule type="cellIs" dxfId="20" priority="1" operator="equal">
       <formula>"0: Environment Setup"</formula>
     </cfRule>
@@ -6754,7 +7400,7 @@
           <x14:formula1>
             <xm:f>Categories!$A$4:$A$25</xm:f>
           </x14:formula1>
-          <xm:sqref>E6:E237</xm:sqref>
+          <xm:sqref>E6:E260</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -6941,11 +7587,11 @@
       </c>
       <c r="D11" s="37">
         <f>SUM(B65)</f>
-        <v>14.75</v>
+        <v>15</v>
       </c>
       <c r="E11" s="38">
         <f t="shared" si="0"/>
-        <v>0.81944444444444442</v>
+        <v>0.83333333333333337</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.3">
@@ -6959,11 +7605,11 @@
       </c>
       <c r="D12" s="54">
         <f>SUM(D5:D11)</f>
-        <v>115.6</v>
+        <v>115.85</v>
       </c>
       <c r="E12" s="55">
         <f>IF(C12=0,0,D12/C12)</f>
-        <v>0.97966101694915253</v>
+        <v>0.98177966101694913</v>
       </c>
     </row>
     <row r="14" spans="1:14" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -7745,7 +8391,7 @@
       </c>
       <c r="B65" s="37">
         <f>SUMIF('Work Log'!E:E,"6: Documentation + Submission",'Work Log'!D:D)</f>
-        <v>14.75</v>
+        <v>15</v>
       </c>
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.3">
@@ -7772,7 +8418,7 @@
       </c>
       <c r="B68" s="93">
         <f>SUM(B46:B67)</f>
-        <v>138.85000000000002</v>
+        <v>139.10000000000002</v>
       </c>
     </row>
   </sheetData>

</xml_diff>